<commit_message>
Publish Loko - Dynamo matchday
</commit_message>
<xml_diff>
--- a/content/src-assets/data/Кубок/cup_128.xlsx
+++ b/content/src-assets/data/Кубок/cup_128.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U69"/>
+  <dimension ref="A1:U68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -531,55 +531,55 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Что это за стадион?</v>
+        <v>За какой из этих европейских клубов играл Андрей Аршавин?</v>
       </c>
       <c r="C3" t="str">
-        <v>std_vtb</v>
+        <v>cup_arshavin</v>
       </c>
       <c r="D3" t="str">
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>std_vtb</v>
+        <v>cup_arshavin</v>
       </c>
       <c r="F3" t="str">
-        <v>logo_dinamo</v>
+        <v>no_pic</v>
       </c>
       <c r="G3" t="str">
-        <v>Динамо Москва</v>
+        <v>Арсенал</v>
       </c>
       <c r="H3" t="str">
-        <v>logo_cska</v>
+        <v>no_pic</v>
       </c>
       <c r="I3" t="str">
-        <v>ЦСКА</v>
+        <v>Ливерпуль</v>
       </c>
       <c r="J3" t="str">
-        <v>logo_spartak</v>
+        <v>no_pic</v>
       </c>
       <c r="K3" t="str">
-        <v>Спартак Москва</v>
+        <v>Манчестер Юнайтед</v>
       </c>
       <c r="L3" t="str">
-        <v>logo_lokomotiv</v>
+        <v>no_pic</v>
       </c>
       <c r="M3" t="str">
-        <v>Локомотив</v>
+        <v>Тоттенхэм</v>
       </c>
       <c r="N3" t="str">
-        <v>logo_zenit</v>
+        <v>no_pic</v>
       </c>
       <c r="O3" t="str">
-        <v>Зенит</v>
+        <v>Эвертон</v>
       </c>
       <c r="P3" t="str">
-        <v>logo_torpedo</v>
+        <v>no_pic</v>
       </c>
       <c r="Q3" t="str">
-        <v>Торпедо Москва</v>
+        <v>Челси</v>
       </c>
       <c r="R3" t="str">
         <v/>
@@ -599,52 +599,52 @@
         <v>1</v>
       </c>
       <c r="B4" t="str">
-        <v>За какой из этих европейских клубов играл Андрей Аршавин?</v>
+        <v>За сколько чемпионств России и СССР клуб может добавить звезду над эмблемой?</v>
       </c>
       <c r="C4" t="str">
-        <v>cup_arshavin</v>
+        <v>no_pic</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>Одна звезда соответствует пяти чемпионским титулам в первенствах СССР и России</v>
       </c>
       <c r="E4" t="str">
-        <v>cup_arshavin</v>
+        <v>no_pic</v>
       </c>
       <c r="F4" t="str">
         <v>no_pic</v>
       </c>
       <c r="G4" t="str">
-        <v>Арсенал</v>
+        <v>5 чемпионств</v>
       </c>
       <c r="H4" t="str">
         <v>no_pic</v>
       </c>
       <c r="I4" t="str">
-        <v>Ливерпуль</v>
+        <v>3 чемпионства</v>
       </c>
       <c r="J4" t="str">
         <v>no_pic</v>
       </c>
       <c r="K4" t="str">
-        <v>Манчестер Юнайтед</v>
+        <v>1 чемпионство</v>
       </c>
       <c r="L4" t="str">
         <v>no_pic</v>
       </c>
       <c r="M4" t="str">
-        <v>Тоттенхэм</v>
+        <v>10 чемпионств</v>
       </c>
       <c r="N4" t="str">
         <v>no_pic</v>
       </c>
       <c r="O4" t="str">
-        <v>Эвертон</v>
+        <v>15 чемпионств</v>
       </c>
       <c r="P4" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q4" t="str">
-        <v>Челси</v>
+        <v>8 чемпионств</v>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -664,52 +664,52 @@
         <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>За сколько чемпионств России и СССР клуб может добавить звезду над эмблемой?</v>
+        <v>Как до 2024 года назывался стадион Лукойл Арена?</v>
       </c>
       <c r="C5" t="str">
-        <v>no_pic</v>
+        <v>std_spartak</v>
       </c>
       <c r="D5" t="str">
-        <v>Одна звезда соответствует пяти чемпионским титулам в первенствах СССР и России</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>no_pic</v>
+        <v>std_spartak</v>
       </c>
       <c r="F5" t="str">
         <v>no_pic</v>
       </c>
       <c r="G5" t="str">
-        <v>5 чемпионств</v>
+        <v>Открытие Банк Арена</v>
       </c>
       <c r="H5" t="str">
         <v>no_pic</v>
       </c>
       <c r="I5" t="str">
-        <v>3 чемпионства</v>
+        <v>Стадион им. Черенкова</v>
       </c>
       <c r="J5" t="str">
         <v>no_pic</v>
       </c>
       <c r="K5" t="str">
-        <v>1 чемпионство</v>
+        <v>Стадион им. Симоняна</v>
       </c>
       <c r="L5" t="str">
         <v>no_pic</v>
       </c>
       <c r="M5" t="str">
-        <v>10 чемпионств</v>
+        <v>Спартак</v>
       </c>
       <c r="N5" t="str">
         <v>no_pic</v>
       </c>
       <c r="O5" t="str">
-        <v>15 чемпионств</v>
+        <v>Волоколамский</v>
       </c>
       <c r="P5" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q5" t="str">
-        <v>8 чемпионств</v>
+        <v>Олимпийский</v>
       </c>
       <c r="R5" t="str">
         <v/>
@@ -729,52 +729,52 @@
         <v>1</v>
       </c>
       <c r="B6" t="str">
-        <v>Как до 2024 года назывался стадион Лукойл Арена?</v>
+        <v>Как зовут главного тренера Зенита?</v>
       </c>
       <c r="C6" t="str">
-        <v>std_spartak</v>
+        <v>zs_semak</v>
       </c>
       <c r="D6" t="str">
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>std_spartak</v>
+        <v>zs_semak</v>
       </c>
       <c r="F6" t="str">
         <v>no_pic</v>
       </c>
       <c r="G6" t="str">
-        <v>Открытие Банк Арена</v>
+        <v>Сергей Семак</v>
       </c>
       <c r="H6" t="str">
         <v>no_pic</v>
       </c>
       <c r="I6" t="str">
-        <v>Стадион им. Черенкова</v>
+        <v>Андрей Талалаев</v>
       </c>
       <c r="J6" t="str">
         <v>no_pic</v>
       </c>
       <c r="K6" t="str">
-        <v>Стадион им. Симоняна</v>
+        <v>Вадим Евсеев</v>
       </c>
       <c r="L6" t="str">
         <v>no_pic</v>
       </c>
       <c r="M6" t="str">
-        <v>Спартак</v>
+        <v>Владимир Федотов</v>
       </c>
       <c r="N6" t="str">
         <v>no_pic</v>
       </c>
       <c r="O6" t="str">
-        <v>Волоколамский</v>
+        <v>Владимир Вайсс</v>
       </c>
       <c r="P6" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q6" t="str">
-        <v>Олимпийский</v>
+        <v>Андрей Тихонов</v>
       </c>
       <c r="R6" t="str">
         <v/>
@@ -794,52 +794,52 @@
         <v>1</v>
       </c>
       <c r="B7" t="str">
-        <v>Как зовут главного тренера Зенита?</v>
+        <v>Как называется стадион Локомотива?</v>
       </c>
       <c r="C7" t="str">
-        <v>zs_semak</v>
+        <v>std_rzd</v>
       </c>
       <c r="D7" t="str">
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>zs_semak</v>
+        <v>std_rzd</v>
       </c>
       <c r="F7" t="str">
         <v>no_pic</v>
       </c>
       <c r="G7" t="str">
-        <v>Сергей Семак</v>
+        <v>РЖД Арена</v>
       </c>
       <c r="H7" t="str">
         <v>no_pic</v>
       </c>
       <c r="I7" t="str">
-        <v>Андрей Талалаев</v>
+        <v>Локомотив Арена</v>
       </c>
       <c r="J7" t="str">
         <v>no_pic</v>
       </c>
       <c r="K7" t="str">
-        <v>Вадим Евсеев</v>
+        <v>Лужники</v>
       </c>
       <c r="L7" t="str">
         <v>no_pic</v>
       </c>
       <c r="M7" t="str">
-        <v>Владимир Федотов</v>
+        <v>Арена Химки</v>
       </c>
       <c r="N7" t="str">
         <v>no_pic</v>
       </c>
       <c r="O7" t="str">
-        <v>Владимир Вайсс</v>
+        <v>Железнодорожный стадион</v>
       </c>
       <c r="P7" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q7" t="str">
-        <v>Андрей Тихонов</v>
+        <v>Стадион им. Лоськова</v>
       </c>
       <c r="R7" t="str">
         <v/>
@@ -859,52 +859,52 @@
         <v>1</v>
       </c>
       <c r="B8" t="str">
-        <v>Как называется стадион Локомотива?</v>
+        <v>Как называется стадион Краснодара?</v>
       </c>
       <c r="C8" t="str">
-        <v>std_rzd</v>
+        <v>std_krasnodar</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>std_rzd</v>
+        <v>std_krasnodar</v>
       </c>
       <c r="F8" t="str">
         <v>no_pic</v>
       </c>
       <c r="G8" t="str">
-        <v>РЖД Арена</v>
+        <v>Ozon Арена</v>
       </c>
       <c r="H8" t="str">
         <v>no_pic</v>
       </c>
       <c r="I8" t="str">
-        <v>Локомотив Арена</v>
+        <v>Кубань</v>
       </c>
       <c r="J8" t="str">
         <v>no_pic</v>
       </c>
       <c r="K8" t="str">
-        <v>Лужники</v>
+        <v>Серп и Молот</v>
       </c>
       <c r="L8" t="str">
         <v>no_pic</v>
       </c>
       <c r="M8" t="str">
-        <v>Арена Химки</v>
+        <v>Краснодар</v>
       </c>
       <c r="N8" t="str">
         <v>no_pic</v>
       </c>
       <c r="O8" t="str">
-        <v>Железнодорожный стадион</v>
+        <v>Стадион им. Галицкого</v>
       </c>
       <c r="P8" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q8" t="str">
-        <v>Стадион им. Лоськова</v>
+        <v>Южный</v>
       </c>
       <c r="R8" t="str">
         <v/>
@@ -924,52 +924,52 @@
         <v>1</v>
       </c>
       <c r="B9" t="str">
-        <v>Как называется стадион Краснодара?</v>
+        <v>Какое животное было официальным талисманом ЧМ-2018?</v>
       </c>
       <c r="C9" t="str">
-        <v>std_krasnodar</v>
+        <v>no_pic</v>
       </c>
       <c r="D9" t="str">
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>std_krasnodar</v>
+        <v>pic_zabivaka</v>
       </c>
       <c r="F9" t="str">
         <v>no_pic</v>
       </c>
       <c r="G9" t="str">
-        <v>Ozon Арена</v>
+        <v>Волк Забивака</v>
       </c>
       <c r="H9" t="str">
         <v>no_pic</v>
       </c>
       <c r="I9" t="str">
-        <v>Кубань</v>
+        <v>Броненосец Фулеко</v>
       </c>
       <c r="J9" t="str">
         <v>no_pic</v>
       </c>
       <c r="K9" t="str">
-        <v>Серп и Молот</v>
+        <v>Медвежонок Миша</v>
       </c>
       <c r="L9" t="str">
         <v>no_pic</v>
       </c>
       <c r="M9" t="str">
-        <v>Краснодар</v>
+        <v>Леопард Лео</v>
       </c>
       <c r="N9" t="str">
         <v>no_pic</v>
       </c>
       <c r="O9" t="str">
-        <v>Стадион им. Галицкого</v>
+        <v>Белый медведь Умка</v>
       </c>
       <c r="P9" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q9" t="str">
-        <v>Южный</v>
+        <v>Заяц Русак</v>
       </c>
       <c r="R9" t="str">
         <v/>
@@ -989,52 +989,52 @@
         <v>1</v>
       </c>
       <c r="B10" t="str">
-        <v>Какое животное было официальным талисманом ЧМ-2018?</v>
+        <v>Какой российский футболист забил четыре мяча «Ливерпулю» на «Энфилде»?</v>
       </c>
       <c r="C10" t="str">
         <v>no_pic</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>21 апреля 2009 года Андрей Аршавин забил четыре мяча «Ливерпулю» в матче Премьер-лиги и стал первым гостевым игроком за 63 года, оформившим покер на «Энфилде»</v>
       </c>
       <c r="E10" t="str">
-        <v>pic_zabivaka</v>
+        <v>cup_arshavin</v>
       </c>
       <c r="F10" t="str">
         <v>no_pic</v>
       </c>
       <c r="G10" t="str">
-        <v>Волк Забивака</v>
+        <v>Андрей Аршавин</v>
       </c>
       <c r="H10" t="str">
         <v>no_pic</v>
       </c>
       <c r="I10" t="str">
-        <v>Броненосец Фулеко</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="J10" t="str">
         <v>no_pic</v>
       </c>
       <c r="K10" t="str">
-        <v>Медвежонок Миша</v>
+        <v>Павел Погребняк</v>
       </c>
       <c r="L10" t="str">
         <v>no_pic</v>
       </c>
       <c r="M10" t="str">
-        <v>Леопард Лео</v>
+        <v>Роман Павлюченко</v>
       </c>
       <c r="N10" t="str">
         <v>no_pic</v>
       </c>
       <c r="O10" t="str">
-        <v>Белый медведь Умка</v>
+        <v>Александр Кержаков</v>
       </c>
       <c r="P10" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q10" t="str">
-        <v>Заяц Русак</v>
+        <v>Артём Дзюба</v>
       </c>
       <c r="R10" t="str">
         <v/>
@@ -1054,52 +1054,52 @@
         <v>1</v>
       </c>
       <c r="B11" t="str">
-        <v>Какой российский футболист забил четыре мяча «Ливерпулю» на «Энфилде»?</v>
+        <v>Какой российский футболист летом 2024 перешёл в ПСЖ?</v>
       </c>
       <c r="C11" t="str">
         <v>no_pic</v>
       </c>
       <c r="D11" t="str">
-        <v>21 апреля 2009 года Андрей Аршавин забил четыре мяча «Ливерпулю» в матче Премьер-лиги и стал первым гостевым игроком за 63 года, оформившим покер на «Энфилде»</v>
+        <v/>
       </c>
       <c r="E11" t="str">
-        <v>cup_arshavin</v>
+        <v>cup_safonov</v>
       </c>
       <c r="F11" t="str">
         <v>no_pic</v>
       </c>
       <c r="G11" t="str">
-        <v>Андрей Аршавин</v>
+        <v>Матвей Сафонов</v>
       </c>
       <c r="H11" t="str">
         <v>no_pic</v>
       </c>
       <c r="I11" t="str">
-        <v>Валерий Карпин</v>
+        <v>Александр Соболев</v>
       </c>
       <c r="J11" t="str">
         <v>no_pic</v>
       </c>
       <c r="K11" t="str">
-        <v>Павел Погребняк</v>
+        <v>Илья Помазун</v>
       </c>
       <c r="L11" t="str">
         <v>no_pic</v>
       </c>
       <c r="M11" t="str">
-        <v>Роман Павлюченко</v>
+        <v>Александр Головин</v>
       </c>
       <c r="N11" t="str">
         <v>no_pic</v>
       </c>
       <c r="O11" t="str">
-        <v>Александр Кержаков</v>
+        <v>Алексей Миранчук</v>
       </c>
       <c r="P11" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q11" t="str">
-        <v>Артём Дзюба</v>
+        <v>Антон Шунин</v>
       </c>
       <c r="R11" t="str">
         <v/>
@@ -1119,7 +1119,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="str">
-        <v>Какой российский футболист летом 2024 перешёл в ПСЖ?</v>
+        <v>Какой российский футболист является воспитанником мадридского Реала?</v>
       </c>
       <c r="C12" t="str">
         <v>no_pic</v>
@@ -1128,43 +1128,43 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>cup_safonov</v>
+        <v>cup_cherishev</v>
       </c>
       <c r="F12" t="str">
         <v>no_pic</v>
       </c>
       <c r="G12" t="str">
-        <v>Матвей Сафонов</v>
+        <v>Денис Черышев</v>
       </c>
       <c r="H12" t="str">
         <v>no_pic</v>
       </c>
       <c r="I12" t="str">
-        <v>Александр Соболев</v>
+        <v>Александр Головин</v>
       </c>
       <c r="J12" t="str">
         <v>no_pic</v>
       </c>
       <c r="K12" t="str">
-        <v>Илья Помазун</v>
+        <v>Алексей Миранчук</v>
       </c>
       <c r="L12" t="str">
         <v>no_pic</v>
       </c>
       <c r="M12" t="str">
-        <v>Александр Головин</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="N12" t="str">
         <v>no_pic</v>
       </c>
       <c r="O12" t="str">
-        <v>Алексей Миранчук</v>
+        <v>Александр Мостовой</v>
       </c>
       <c r="P12" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q12" t="str">
-        <v>Антон Шунин</v>
+        <v>Дмитрий Черышев</v>
       </c>
       <c r="R12" t="str">
         <v/>
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="B13" t="str">
-        <v>Какой российский футболист является воспитанником мадридского Реала?</v>
+        <v>Какой советский вратарь в своё время получил Золотой Мяч?</v>
       </c>
       <c r="C13" t="str">
         <v>no_pic</v>
@@ -1193,43 +1193,43 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>cup_cherishev</v>
+        <v>cup_yashin</v>
       </c>
       <c r="F13" t="str">
         <v>no_pic</v>
       </c>
       <c r="G13" t="str">
-        <v>Денис Черышев</v>
+        <v>Лев Яшин</v>
       </c>
       <c r="H13" t="str">
         <v>no_pic</v>
       </c>
       <c r="I13" t="str">
-        <v>Александр Головин</v>
+        <v>Станислав Черчесов</v>
       </c>
       <c r="J13" t="str">
         <v>no_pic</v>
       </c>
       <c r="K13" t="str">
-        <v>Алексей Миранчук</v>
+        <v>Ринат Дасаев</v>
       </c>
       <c r="L13" t="str">
         <v>no_pic</v>
       </c>
       <c r="M13" t="str">
-        <v>Валерий Карпин</v>
+        <v>Владимир Маслаченко</v>
       </c>
       <c r="N13" t="str">
         <v>no_pic</v>
       </c>
       <c r="O13" t="str">
-        <v>Александр Мостовой</v>
+        <v>Владимир Пильгуй</v>
       </c>
       <c r="P13" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q13" t="str">
-        <v>Дмитрий Черышев</v>
+        <v>Руслан Нигматуллин</v>
       </c>
       <c r="R13" t="str">
         <v/>
@@ -1249,7 +1249,7 @@
         <v>1</v>
       </c>
       <c r="B14" t="str">
-        <v>Какой советский вратарь в своё время получил Золотой Мяч?</v>
+        <v>Кому принадлежит фраза "Ваши ожидания - Ваши проблемы"?</v>
       </c>
       <c r="C14" t="str">
         <v>no_pic</v>
@@ -1258,43 +1258,43 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>cup_yashin</v>
+        <v>cup_arshavin</v>
       </c>
       <c r="F14" t="str">
         <v>no_pic</v>
       </c>
       <c r="G14" t="str">
-        <v>Лев Яшин</v>
+        <v>Андрей Аршавин</v>
       </c>
       <c r="H14" t="str">
         <v>no_pic</v>
       </c>
       <c r="I14" t="str">
+        <v>Александр Кержаков</v>
+      </c>
+      <c r="J14" t="str">
+        <v>no_pic</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Артём Дзюба</v>
+      </c>
+      <c r="L14" t="str">
+        <v>no_pic</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Валерий Карпин</v>
+      </c>
+      <c r="N14" t="str">
+        <v>no_pic</v>
+      </c>
+      <c r="O14" t="str">
         <v>Станислав Черчесов</v>
       </c>
-      <c r="J14" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Ринат Дасаев</v>
-      </c>
-      <c r="L14" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="M14" t="str">
-        <v>Владимир Маслаченко</v>
-      </c>
-      <c r="N14" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="O14" t="str">
-        <v>Владимир Пильгуй</v>
-      </c>
       <c r="P14" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q14" t="str">
-        <v>Руслан Нигматуллин</v>
+        <v>Фабио Капелло</v>
       </c>
       <c r="R14" t="str">
         <v/>
@@ -1314,52 +1314,52 @@
         <v>1</v>
       </c>
       <c r="B15" t="str">
-        <v>Кому принадлежит фраза "Ваши ожидания - Ваши проблемы"?</v>
+        <v>Кого в 2012 году Артём Дзюба, играя за Спартак, назвал "трениришкой"?</v>
       </c>
       <c r="C15" t="str">
-        <v>no_pic</v>
+        <v>cup_dzyba</v>
       </c>
       <c r="D15" t="str">
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>cup_arshavin</v>
+        <v>logo_spartak</v>
       </c>
       <c r="F15" t="str">
         <v>no_pic</v>
       </c>
       <c r="G15" t="str">
-        <v>Андрей Аршавин</v>
+        <v>Унаи Эмери</v>
       </c>
       <c r="H15" t="str">
         <v>no_pic</v>
       </c>
       <c r="I15" t="str">
-        <v>Александр Кержаков</v>
+        <v>Руй Витория</v>
       </c>
       <c r="J15" t="str">
         <v>no_pic</v>
       </c>
       <c r="K15" t="str">
-        <v>Артём Дзюба</v>
+        <v xml:space="preserve">Рауль Рианчо </v>
       </c>
       <c r="L15" t="str">
         <v>no_pic</v>
       </c>
       <c r="M15" t="str">
-        <v>Валерий Карпин</v>
+        <v>Мурат Якин</v>
       </c>
       <c r="N15" t="str">
         <v>no_pic</v>
       </c>
       <c r="O15" t="str">
-        <v>Станислав Черчесов</v>
+        <v>Невио Скала</v>
       </c>
       <c r="P15" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q15" t="str">
-        <v>Фабио Капелло</v>
+        <v xml:space="preserve">Массимо Каррера </v>
       </c>
       <c r="R15" t="str">
         <v/>
@@ -1379,52 +1379,52 @@
         <v>1</v>
       </c>
       <c r="B16" t="str">
-        <v>Кого в 2012 году Артём Дзюба, играя за Спартак, назвал "трениришкой"?</v>
+        <v>Кто автор пента-трика в матче Чемпионата Мира 1994 года за сборную России?</v>
       </c>
       <c r="C16" t="str">
-        <v>cup_dzyba</v>
+        <v>no_pic</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>logo_spartak</v>
+        <v>cup_saenko</v>
       </c>
       <c r="F16" t="str">
         <v>no_pic</v>
       </c>
       <c r="G16" t="str">
-        <v>Унаи Эмери</v>
+        <v>Олег Саленко</v>
       </c>
       <c r="H16" t="str">
         <v>no_pic</v>
       </c>
       <c r="I16" t="str">
-        <v>Руй Витория</v>
+        <v>Владимир Бесчастных</v>
       </c>
       <c r="J16" t="str">
         <v>no_pic</v>
       </c>
       <c r="K16" t="str">
-        <v xml:space="preserve">Рауль Рианчо </v>
+        <v>Александр Бородюк</v>
       </c>
       <c r="L16" t="str">
         <v>no_pic</v>
       </c>
       <c r="M16" t="str">
-        <v>Мурат Якин</v>
+        <v>Александр Мостовой</v>
       </c>
       <c r="N16" t="str">
         <v>no_pic</v>
       </c>
       <c r="O16" t="str">
-        <v>Невио Скала</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="P16" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q16" t="str">
-        <v xml:space="preserve">Массимо Каррера </v>
+        <v>Сергей Юран</v>
       </c>
       <c r="R16" t="str">
         <v/>
@@ -1444,7 +1444,7 @@
         <v>1</v>
       </c>
       <c r="B17" t="str">
-        <v>Кто автор пента-трика в матче Чемпионата Мира 1994 года за сборную России?</v>
+        <v>Кто был основным вратарём сборной России на ЧМ-2018?</v>
       </c>
       <c r="C17" t="str">
         <v>no_pic</v>
@@ -1453,43 +1453,43 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>cup_saenko</v>
+        <v>cska_akinfeev</v>
       </c>
       <c r="F17" t="str">
         <v>no_pic</v>
       </c>
       <c r="G17" t="str">
-        <v>Олег Саленко</v>
+        <v>Игорь Акинфеев</v>
       </c>
       <c r="H17" t="str">
         <v>no_pic</v>
       </c>
       <c r="I17" t="str">
-        <v>Владимир Бесчастных</v>
+        <v>Антон Шунин</v>
       </c>
       <c r="J17" t="str">
         <v>no_pic</v>
       </c>
       <c r="K17" t="str">
-        <v>Александр Бородюк</v>
+        <v>Матвей Сафонов</v>
       </c>
       <c r="L17" t="str">
         <v>no_pic</v>
       </c>
       <c r="M17" t="str">
-        <v>Александр Мостовой</v>
+        <v>Владимир Габулов</v>
       </c>
       <c r="N17" t="str">
         <v>no_pic</v>
       </c>
       <c r="O17" t="str">
-        <v>Валерий Карпин</v>
+        <v>Юрий Лодыгин</v>
       </c>
       <c r="P17" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q17" t="str">
-        <v>Сергей Юран</v>
+        <v>Андрей Лунёв</v>
       </c>
       <c r="R17" t="str">
         <v/>
@@ -1509,7 +1509,7 @@
         <v>1</v>
       </c>
       <c r="B18" t="str">
-        <v>Кто был основным вратарём сборной России на ЧМ-2018?</v>
+        <v>Кто был тренером сборной России на ЧМ-2018?</v>
       </c>
       <c r="C18" t="str">
         <v>no_pic</v>
@@ -1518,43 +1518,43 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>cska_akinfeev</v>
+        <v>akhmat_cherchesov</v>
       </c>
       <c r="F18" t="str">
         <v>no_pic</v>
       </c>
       <c r="G18" t="str">
-        <v>Игорь Акинфеев</v>
+        <v>Станислав Черчесов</v>
       </c>
       <c r="H18" t="str">
         <v>no_pic</v>
       </c>
       <c r="I18" t="str">
-        <v>Антон Шунин</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="J18" t="str">
         <v>no_pic</v>
       </c>
       <c r="K18" t="str">
-        <v>Матвей Сафонов</v>
+        <v>Леонид Слуцкий</v>
       </c>
       <c r="L18" t="str">
         <v>no_pic</v>
       </c>
       <c r="M18" t="str">
-        <v>Владимир Габулов</v>
+        <v>Фабио Капелло</v>
       </c>
       <c r="N18" t="str">
         <v>no_pic</v>
       </c>
       <c r="O18" t="str">
-        <v>Юрий Лодыгин</v>
+        <v>Гус Хиддинк</v>
       </c>
       <c r="P18" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q18" t="str">
-        <v>Андрей Лунёв</v>
+        <v>Дик Адвокат</v>
       </c>
       <c r="R18" t="str">
         <v/>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="B19" t="str">
-        <v>Кто был тренером сборной России на ЧМ-2018?</v>
+        <v>Кто из российских футболистов играл и забивал в финалах Лиги Чемпионов и Кубка УЕФА?</v>
       </c>
       <c r="C19" t="str">
         <v>no_pic</v>
@@ -1583,43 +1583,43 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>akhmat_cherchesov</v>
+        <v>cup_alenichev</v>
       </c>
       <c r="F19" t="str">
         <v>no_pic</v>
       </c>
       <c r="G19" t="str">
-        <v>Станислав Черчесов</v>
+        <v>Дмитрий Аленичев</v>
       </c>
       <c r="H19" t="str">
         <v>no_pic</v>
       </c>
       <c r="I19" t="str">
-        <v>Валерий Карпин</v>
+        <v>Сергей Семак</v>
       </c>
       <c r="J19" t="str">
         <v>no_pic</v>
       </c>
       <c r="K19" t="str">
-        <v>Леонид Слуцкий</v>
+        <v>Андрей Аршавин</v>
       </c>
       <c r="L19" t="str">
         <v>no_pic</v>
       </c>
       <c r="M19" t="str">
-        <v>Фабио Капелло</v>
+        <v>Павел Погребняк</v>
       </c>
       <c r="N19" t="str">
         <v>no_pic</v>
       </c>
       <c r="O19" t="str">
-        <v>Гус Хиддинк</v>
+        <v>Денис Черышев</v>
       </c>
       <c r="P19" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q19" t="str">
-        <v>Дик Адвокат</v>
+        <v>Александр Головин</v>
       </c>
       <c r="R19" t="str">
         <v/>
@@ -1639,7 +1639,7 @@
         <v>1</v>
       </c>
       <c r="B20" t="str">
-        <v>Кто из российских футболистов играл и забивал в финалах Лиги Чемпионов и Кубка УЕФА?</v>
+        <v>Кто из этих тренеров никогда не возглавлял сборную России по футболу?</v>
       </c>
       <c r="C20" t="str">
         <v>no_pic</v>
@@ -1648,43 +1648,43 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>cup_alenichev</v>
+        <v>no_pic</v>
       </c>
       <c r="F20" t="str">
         <v>no_pic</v>
       </c>
       <c r="G20" t="str">
-        <v>Дмитрий Аленичев</v>
+        <v>Курбан Бердыев</v>
       </c>
       <c r="H20" t="str">
         <v>no_pic</v>
       </c>
       <c r="I20" t="str">
-        <v>Сергей Семак</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="J20" t="str">
         <v>no_pic</v>
       </c>
       <c r="K20" t="str">
-        <v>Андрей Аршавин</v>
+        <v>Леонид Слуцкий</v>
       </c>
       <c r="L20" t="str">
         <v>no_pic</v>
       </c>
       <c r="M20" t="str">
-        <v>Павел Погребняк</v>
+        <v>Станислав Черчесов</v>
       </c>
       <c r="N20" t="str">
         <v>no_pic</v>
       </c>
       <c r="O20" t="str">
-        <v>Денис Черышев</v>
+        <v>Юрий Сёмин</v>
       </c>
       <c r="P20" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q20" t="str">
-        <v>Александр Головин</v>
+        <v>Дик Адвокат</v>
       </c>
       <c r="R20" t="str">
         <v/>
@@ -1704,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="B21" t="str">
-        <v>Кто из этих тренеров никогда не возглавлял сборную России по футболу?</v>
+        <v>Кто из этих футболистов выигрывал Лигу Чемпионов?</v>
       </c>
       <c r="C21" t="str">
         <v>no_pic</v>
@@ -1713,43 +1713,43 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>no_pic</v>
+        <v>cup_cherishev</v>
       </c>
       <c r="F21" t="str">
         <v>no_pic</v>
       </c>
       <c r="G21" t="str">
-        <v>Курбан Бердыев</v>
+        <v>Денис Черышев</v>
       </c>
       <c r="H21" t="str">
         <v>no_pic</v>
       </c>
       <c r="I21" t="str">
+        <v>Игорь Акинфеев</v>
+      </c>
+      <c r="J21" t="str">
+        <v>no_pic</v>
+      </c>
+      <c r="K21" t="str">
         <v>Валерий Карпин</v>
       </c>
-      <c r="J21" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="K21" t="str">
-        <v>Леонид Слуцкий</v>
-      </c>
       <c r="L21" t="str">
         <v>no_pic</v>
       </c>
       <c r="M21" t="str">
-        <v>Станислав Черчесов</v>
+        <v>Александр Мостовой</v>
       </c>
       <c r="N21" t="str">
         <v>no_pic</v>
       </c>
       <c r="O21" t="str">
-        <v>Юрий Сёмин</v>
+        <v>Роман Павлюченко</v>
       </c>
       <c r="P21" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q21" t="str">
-        <v>Дик Адвокат</v>
+        <v>Павел Погребняк</v>
       </c>
       <c r="R21" t="str">
         <v/>
@@ -1769,7 +1769,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="str">
-        <v>Кто из этих футболистов выигрывал Лигу Чемпионов?</v>
+        <v>Кто из этих футболистов играл и за Зенит, и за Динамо?</v>
       </c>
       <c r="C22" t="str">
         <v>no_pic</v>
@@ -1778,43 +1778,43 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>cup_cherishev</v>
+        <v>no_pic</v>
       </c>
       <c r="F22" t="str">
         <v>no_pic</v>
       </c>
       <c r="G22" t="str">
-        <v>Денис Черышев</v>
+        <v>Александр Кокорин</v>
       </c>
       <c r="H22" t="str">
         <v>no_pic</v>
       </c>
       <c r="I22" t="str">
-        <v>Игорь Акинфеев</v>
+        <v>Александр Анюков</v>
       </c>
       <c r="J22" t="str">
         <v>no_pic</v>
       </c>
       <c r="K22" t="str">
-        <v>Валерий Карпин</v>
+        <v>Роман Широков</v>
       </c>
       <c r="L22" t="str">
         <v>no_pic</v>
       </c>
       <c r="M22" t="str">
-        <v>Александр Мостовой</v>
+        <v>Роман Павлюченко</v>
       </c>
       <c r="N22" t="str">
         <v>no_pic</v>
       </c>
       <c r="O22" t="str">
-        <v>Роман Павлюченко</v>
+        <v>Дмитрий Тарасов</v>
       </c>
       <c r="P22" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q22" t="str">
-        <v>Павел Погребняк</v>
+        <v>Дмитрий Аленичев</v>
       </c>
       <c r="R22" t="str">
         <v/>
@@ -1834,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="B23" t="str">
-        <v>Кто из этих футболистов играл и за Зенит, и за Динамо?</v>
+        <v>Кто из этих футболистов играл и за Зенит, и за ЦСКА?</v>
       </c>
       <c r="C23" t="str">
         <v>no_pic</v>
@@ -1849,37 +1849,37 @@
         <v>no_pic</v>
       </c>
       <c r="G23" t="str">
-        <v>Александр Кокорин</v>
+        <v>Юрий Жирков</v>
       </c>
       <c r="H23" t="str">
         <v>no_pic</v>
       </c>
       <c r="I23" t="str">
-        <v>Александр Анюков</v>
+        <v>Николас Ломбертс</v>
       </c>
       <c r="J23" t="str">
         <v>no_pic</v>
       </c>
       <c r="K23" t="str">
-        <v>Роман Широков</v>
+        <v>Олег Шатов</v>
       </c>
       <c r="L23" t="str">
         <v>no_pic</v>
       </c>
       <c r="M23" t="str">
-        <v>Роман Павлюченко</v>
+        <v>Жулиано</v>
       </c>
       <c r="N23" t="str">
         <v>no_pic</v>
       </c>
       <c r="O23" t="str">
-        <v>Дмитрий Тарасов</v>
+        <v>Роберт Мак</v>
       </c>
       <c r="P23" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q23" t="str">
-        <v>Дмитрий Аленичев</v>
+        <v>Сергей Петров</v>
       </c>
       <c r="R23" t="str">
         <v/>
@@ -1899,52 +1899,52 @@
         <v>1</v>
       </c>
       <c r="B24" t="str">
-        <v>Кто из этих футболистов играл и за Зенит, и за ЦСКА?</v>
+        <v>Кто этот футболист?</v>
       </c>
       <c r="C24" t="str">
-        <v>no_pic</v>
+        <v>spartak_zobnin</v>
       </c>
       <c r="D24" t="str">
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>no_pic</v>
+        <v>spartak_zobnin</v>
       </c>
       <c r="F24" t="str">
         <v>no_pic</v>
       </c>
       <c r="G24" t="str">
-        <v>Юрий Жирков</v>
+        <v>Роман Зобнин</v>
       </c>
       <c r="H24" t="str">
         <v>no_pic</v>
       </c>
       <c r="I24" t="str">
-        <v>Николас Ломбертс</v>
+        <v>Данил Пруцев</v>
       </c>
       <c r="J24" t="str">
         <v>no_pic</v>
       </c>
       <c r="K24" t="str">
-        <v>Олег Шатов</v>
+        <v>Павел Мелешин</v>
       </c>
       <c r="L24" t="str">
         <v>no_pic</v>
       </c>
       <c r="M24" t="str">
-        <v>Жулиано</v>
+        <v>Срджан Бабич</v>
       </c>
       <c r="N24" t="str">
         <v>no_pic</v>
       </c>
       <c r="O24" t="str">
-        <v>Роберт Мак</v>
+        <v xml:space="preserve"> Никита Чернов</v>
       </c>
       <c r="P24" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q24" t="str">
-        <v>Сергей Петров</v>
+        <v>Михаил Игнатов</v>
       </c>
       <c r="R24" t="str">
         <v/>
@@ -1967,49 +1967,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C25" t="str">
-        <v>spartak_zobnin</v>
+        <v>cska_akinfeev</v>
       </c>
       <c r="D25" t="str">
         <v/>
       </c>
       <c r="E25" t="str">
-        <v>spartak_zobnin</v>
+        <v>cska_akinfeev</v>
       </c>
       <c r="F25" t="str">
         <v>no_pic</v>
       </c>
       <c r="G25" t="str">
-        <v>Роман Зобнин</v>
+        <v>Игорь Акинфеев</v>
       </c>
       <c r="H25" t="str">
         <v>no_pic</v>
       </c>
       <c r="I25" t="str">
-        <v>Данил Пруцев</v>
+        <v>Игорь Дивеев</v>
       </c>
       <c r="J25" t="str">
         <v>no_pic</v>
       </c>
       <c r="K25" t="str">
-        <v>Павел Мелешин</v>
+        <v>Владислав Тороп</v>
       </c>
       <c r="L25" t="str">
         <v>no_pic</v>
       </c>
       <c r="M25" t="str">
-        <v>Срджан Бабич</v>
+        <v>Илья Помазун</v>
       </c>
       <c r="N25" t="str">
         <v>no_pic</v>
       </c>
       <c r="O25" t="str">
-        <v xml:space="preserve"> Никита Чернов</v>
+        <v>Николай Баровский</v>
       </c>
       <c r="P25" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q25" t="str">
-        <v>Михаил Игнатов</v>
+        <v>Вадим Конюхов</v>
       </c>
       <c r="R25" t="str">
         <v/>
@@ -2032,49 +2032,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C26" t="str">
-        <v>cska_akinfeev</v>
+        <v>dinamo_tyukavin</v>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>cska_akinfeev</v>
+        <v>dinamo_tyukavin</v>
       </c>
       <c r="F26" t="str">
         <v>no_pic</v>
       </c>
       <c r="G26" t="str">
-        <v>Игорь Акинфеев</v>
+        <v>Константин Тюкавин</v>
       </c>
       <c r="H26" t="str">
         <v>no_pic</v>
       </c>
       <c r="I26" t="str">
-        <v>Игорь Дивеев</v>
+        <v>Александр Кутицкий</v>
       </c>
       <c r="J26" t="str">
         <v>no_pic</v>
       </c>
       <c r="K26" t="str">
-        <v>Владислав Тороп</v>
+        <v>Максим Александров</v>
       </c>
       <c r="L26" t="str">
         <v>no_pic</v>
       </c>
       <c r="M26" t="str">
-        <v>Илья Помазун</v>
+        <v>Даниил Лесовой</v>
       </c>
       <c r="N26" t="str">
         <v>no_pic</v>
       </c>
       <c r="O26" t="str">
-        <v>Николай Баровский</v>
+        <v>Александр Чупаев</v>
       </c>
       <c r="P26" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q26" t="str">
-        <v>Вадим Конюхов</v>
+        <v>Курбан Расулов</v>
       </c>
       <c r="R26" t="str">
         <v/>
@@ -2097,49 +2097,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C27" t="str">
-        <v>dinamo_tyukavin</v>
+        <v>cska_barinov</v>
       </c>
       <c r="D27" t="str">
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>dinamo_tyukavin</v>
+        <v>cska_barinov</v>
       </c>
       <c r="F27" t="str">
         <v>no_pic</v>
       </c>
       <c r="G27" t="str">
-        <v>Константин Тюкавин</v>
+        <v>Дмитрий Баринов</v>
       </c>
       <c r="H27" t="str">
         <v>no_pic</v>
       </c>
       <c r="I27" t="str">
-        <v>Александр Кутицкий</v>
+        <v>Максим Ненахов</v>
       </c>
       <c r="J27" t="str">
         <v>no_pic</v>
       </c>
       <c r="K27" t="str">
-        <v>Максим Александров</v>
+        <v>Алексей Батраков</v>
       </c>
       <c r="L27" t="str">
         <v>no_pic</v>
       </c>
       <c r="M27" t="str">
-        <v>Даниил Лесовой</v>
+        <v>Тимур Сулейманов</v>
       </c>
       <c r="N27" t="str">
         <v>no_pic</v>
       </c>
       <c r="O27" t="str">
-        <v>Александр Чупаев</v>
+        <v>Владислав Сарвели</v>
       </c>
       <c r="P27" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q27" t="str">
-        <v>Курбан Расулов</v>
+        <v>Илья Лантратов</v>
       </c>
       <c r="R27" t="str">
         <v/>
@@ -2162,49 +2162,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C28" t="str">
-        <v>cska_barinov</v>
+        <v>cup_smolov</v>
       </c>
       <c r="D28" t="str">
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>cska_barinov</v>
+        <v>cup_smolov</v>
       </c>
       <c r="F28" t="str">
         <v>no_pic</v>
       </c>
       <c r="G28" t="str">
-        <v>Дмитрий Баринов</v>
+        <v>Федор Смолов</v>
       </c>
       <c r="H28" t="str">
         <v>no_pic</v>
       </c>
       <c r="I28" t="str">
-        <v>Максим Ненахов</v>
+        <v>Сергей Петров</v>
       </c>
       <c r="J28" t="str">
         <v>no_pic</v>
       </c>
       <c r="K28" t="str">
-        <v>Алексей Батраков</v>
+        <v>Юрий Дюпин</v>
       </c>
       <c r="L28" t="str">
         <v>no_pic</v>
       </c>
       <c r="M28" t="str">
-        <v>Тимур Сулейманов</v>
+        <v>Станислав Агкацев</v>
       </c>
       <c r="N28" t="str">
         <v>no_pic</v>
       </c>
       <c r="O28" t="str">
-        <v>Владислав Сарвели</v>
+        <v>Александр Черников</v>
       </c>
       <c r="P28" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q28" t="str">
-        <v>Илья Лантратов</v>
+        <v>Александр Кокшаров</v>
       </c>
       <c r="R28" t="str">
         <v/>
@@ -2224,52 +2224,52 @@
         <v>1</v>
       </c>
       <c r="B29" t="str">
-        <v>Кто этот футболист?</v>
+        <v>Кто является бессменным президентом и владельцем Краснодара?</v>
       </c>
       <c r="C29" t="str">
-        <v>cup_smolov</v>
+        <v>no_pic</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>Сергей Галицкий является президентом и владельцем Краснодара с момента основания клуба</v>
       </c>
       <c r="E29" t="str">
-        <v>cup_smolov</v>
+        <v>logo_krasnodar</v>
       </c>
       <c r="F29" t="str">
         <v>no_pic</v>
       </c>
       <c r="G29" t="str">
-        <v>Федор Смолов</v>
+        <v>Сергей Галицкий</v>
       </c>
       <c r="H29" t="str">
         <v>no_pic</v>
       </c>
       <c r="I29" t="str">
-        <v>Сергей Петров</v>
+        <v>Павел Пивоваров</v>
       </c>
       <c r="J29" t="str">
         <v>no_pic</v>
       </c>
       <c r="K29" t="str">
-        <v>Юрий Дюпин</v>
+        <v>Николай Толстых</v>
       </c>
       <c r="L29" t="str">
         <v>no_pic</v>
       </c>
       <c r="M29" t="str">
-        <v>Станислав Агкацев</v>
+        <v>Валерий Бубнов</v>
       </c>
       <c r="N29" t="str">
         <v>no_pic</v>
       </c>
       <c r="O29" t="str">
-        <v>Александр Черников</v>
+        <v>Арам Фундукян</v>
       </c>
       <c r="P29" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q29" t="str">
-        <v>Александр Кокшаров</v>
+        <v>Аслан Засеев</v>
       </c>
       <c r="R29" t="str">
         <v/>
@@ -2286,55 +2286,55 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" t="str">
-        <v>Кто является бессменным президентом и владельцем Краснодара?</v>
+        <v>На каком стадионе был сыгран финал Чемпионата Мира по футболу 2018?</v>
       </c>
       <c r="C30" t="str">
         <v>no_pic</v>
       </c>
       <c r="D30" t="str">
-        <v>Сергей Галицкий является президентом и владельцем Краснодара с момента основания клуба</v>
+        <v/>
       </c>
       <c r="E30" t="str">
-        <v>logo_krasnodar</v>
+        <v>std_lujniki</v>
       </c>
       <c r="F30" t="str">
-        <v>no_pic</v>
+        <v>std_lujniki</v>
       </c>
       <c r="G30" t="str">
-        <v>Сергей Галицкий</v>
+        <v>Лужники</v>
       </c>
       <c r="H30" t="str">
-        <v>no_pic</v>
+        <v>std_nizhnov</v>
       </c>
       <c r="I30" t="str">
-        <v>Павел Пивоваров</v>
+        <v>Нижний Новгород</v>
       </c>
       <c r="J30" t="str">
-        <v>no_pic</v>
+        <v>std_spartak</v>
       </c>
       <c r="K30" t="str">
-        <v>Николай Толстых</v>
+        <v>Лукойл Арена</v>
       </c>
       <c r="L30" t="str">
-        <v>no_pic</v>
+        <v>std_krasnodar</v>
       </c>
       <c r="M30" t="str">
-        <v>Валерий Бубнов</v>
+        <v>Краснодар</v>
       </c>
       <c r="N30" t="str">
-        <v>no_pic</v>
+        <v>std_rzd</v>
       </c>
       <c r="O30" t="str">
-        <v>Арам Фундукян</v>
+        <v>РЖД Арена</v>
       </c>
       <c r="P30" t="str">
-        <v>no_pic</v>
+        <v>std_vtb</v>
       </c>
       <c r="Q30" t="str">
-        <v>Аслан Засеев</v>
+        <v>ВТБ Арена</v>
       </c>
       <c r="R30" t="str">
         <v/>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B31" t="str">
-        <v>На каком стадионе был сыгран финал Чемпионата Мира по футболу 2018?</v>
+        <v>На слиянии каких рек находится домашний стадион ФК "Нижний Новгород"?</v>
       </c>
       <c r="C31" t="str">
         <v>no_pic</v>
@@ -2363,43 +2363,43 @@
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>std_lujniki</v>
+        <v>std_nizhnov</v>
       </c>
       <c r="F31" t="str">
-        <v>std_lujniki</v>
+        <v>no_pic</v>
       </c>
       <c r="G31" t="str">
-        <v>Лужники</v>
+        <v>Волга и Ока</v>
       </c>
       <c r="H31" t="str">
-        <v>std_nizhnov</v>
+        <v>no_pic</v>
       </c>
       <c r="I31" t="str">
-        <v>Нижний Новгород</v>
+        <v>Волга и Обь</v>
       </c>
       <c r="J31" t="str">
-        <v>std_spartak</v>
+        <v>no_pic</v>
       </c>
       <c r="K31" t="str">
-        <v>Лукойл Арена</v>
+        <v>Волга и Кама</v>
       </c>
       <c r="L31" t="str">
-        <v>std_krasnodar</v>
+        <v>no_pic</v>
       </c>
       <c r="M31" t="str">
-        <v>Краснодар</v>
+        <v>Волга и Аргунь</v>
       </c>
       <c r="N31" t="str">
-        <v>std_rzd</v>
+        <v>no_pic</v>
       </c>
       <c r="O31" t="str">
-        <v>РЖД Арена</v>
+        <v>Волга и Иртыш</v>
       </c>
       <c r="P31" t="str">
-        <v>std_vtb</v>
+        <v>no_pic</v>
       </c>
       <c r="Q31" t="str">
-        <v>ВТБ Арена</v>
+        <v>Волга и Дон</v>
       </c>
       <c r="R31" t="str">
         <v/>
@@ -2419,7 +2419,7 @@
         <v>1</v>
       </c>
       <c r="B32" t="str">
-        <v>На слиянии каких рек находится домашний стадион ФК "Нижний Новгород"?</v>
+        <v>До какой стадии сборная России доходила на чемпионатах Европы?</v>
       </c>
       <c r="C32" t="str">
         <v>no_pic</v>
@@ -2428,43 +2428,43 @@
         <v/>
       </c>
       <c r="E32" t="str">
-        <v>std_nizhnov</v>
+        <v>no_pic</v>
       </c>
       <c r="F32" t="str">
         <v>no_pic</v>
       </c>
       <c r="G32" t="str">
-        <v>Волга и Ока</v>
+        <v>Полуфинал</v>
       </c>
       <c r="H32" t="str">
         <v>no_pic</v>
       </c>
       <c r="I32" t="str">
-        <v>Волга и Обь</v>
+        <v>2 место</v>
       </c>
       <c r="J32" t="str">
         <v>no_pic</v>
       </c>
       <c r="K32" t="str">
-        <v>Волга и Кама</v>
+        <v>Четвертьфинал</v>
       </c>
       <c r="L32" t="str">
         <v>no_pic</v>
       </c>
       <c r="M32" t="str">
-        <v>Волга и Аргунь</v>
+        <v>Групповой этап</v>
       </c>
       <c r="N32" t="str">
         <v>no_pic</v>
       </c>
       <c r="O32" t="str">
-        <v>Волга и Иртыш</v>
+        <v>1/8 финала</v>
       </c>
       <c r="P32" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="Q32" t="str">
-        <v>Волга и Дон</v>
+        <v/>
       </c>
       <c r="R32" t="str">
         <v/>
@@ -2484,7 +2484,7 @@
         <v>1</v>
       </c>
       <c r="B33" t="str">
-        <v>До какой стадии сборная России доходила на чемпионатах Европы?</v>
+        <v>От какой сборной Игорь Акинфеев пропустил курьезный гол на ЧМ-2014?</v>
       </c>
       <c r="C33" t="str">
         <v>no_pic</v>
@@ -2499,37 +2499,37 @@
         <v>no_pic</v>
       </c>
       <c r="G33" t="str">
-        <v>Полуфинал</v>
+        <v>Южная Корея</v>
       </c>
       <c r="H33" t="str">
         <v>no_pic</v>
       </c>
       <c r="I33" t="str">
-        <v>2 место</v>
+        <v>Алжир</v>
       </c>
       <c r="J33" t="str">
         <v>no_pic</v>
       </c>
       <c r="K33" t="str">
-        <v>Четвертьфинал</v>
+        <v>Бельгия</v>
       </c>
       <c r="L33" t="str">
         <v>no_pic</v>
       </c>
       <c r="M33" t="str">
-        <v>Групповой этап</v>
+        <v>Япония</v>
       </c>
       <c r="N33" t="str">
         <v>no_pic</v>
       </c>
       <c r="O33" t="str">
-        <v>1/8 финала</v>
+        <v>Мексика</v>
       </c>
       <c r="P33" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="Q33" t="str">
-        <v/>
+        <v>Уэльс</v>
       </c>
       <c r="R33" t="str">
         <v/>
@@ -2549,52 +2549,52 @@
         <v>1</v>
       </c>
       <c r="B34" t="str">
-        <v>От какой сборной Игорь Акинфеев пропустил курьезный гол на ЧМ-2014?</v>
+        <v>Чья эта эмблема?</v>
       </c>
       <c r="C34" t="str">
-        <v>no_pic</v>
+        <v>logo_rubin_t</v>
       </c>
       <c r="D34" t="str">
         <v/>
       </c>
       <c r="E34" t="str">
-        <v>no_pic</v>
+        <v>logo_rubin</v>
       </c>
       <c r="F34" t="str">
         <v>no_pic</v>
       </c>
       <c r="G34" t="str">
-        <v>Южная Корея</v>
+        <v>Рубин</v>
       </c>
       <c r="H34" t="str">
         <v>no_pic</v>
       </c>
       <c r="I34" t="str">
-        <v>Алжир</v>
+        <v>Ростов</v>
       </c>
       <c r="J34" t="str">
         <v>no_pic</v>
       </c>
       <c r="K34" t="str">
-        <v>Бельгия</v>
+        <v>Ротор</v>
       </c>
       <c r="L34" t="str">
         <v>no_pic</v>
       </c>
       <c r="M34" t="str">
-        <v>Япония</v>
+        <v>Сочи</v>
       </c>
       <c r="N34" t="str">
         <v>no_pic</v>
       </c>
       <c r="O34" t="str">
-        <v>Мексика</v>
+        <v>Акрон</v>
       </c>
       <c r="P34" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q34" t="str">
-        <v>Уэльс</v>
+        <v>Ахмат</v>
       </c>
       <c r="R34" t="str">
         <v/>
@@ -2617,49 +2617,49 @@
         <v>Чья эта эмблема?</v>
       </c>
       <c r="C35" t="str">
-        <v>logo_rubin_t</v>
+        <v>logo_ks</v>
       </c>
       <c r="D35" t="str">
         <v/>
       </c>
       <c r="E35" t="str">
-        <v>logo_rubin</v>
+        <v>logo_ks</v>
       </c>
       <c r="F35" t="str">
         <v>no_pic</v>
       </c>
       <c r="G35" t="str">
-        <v>Рубин</v>
+        <v>Крылья Советов</v>
       </c>
       <c r="H35" t="str">
         <v>no_pic</v>
       </c>
       <c r="I35" t="str">
-        <v>Ростов</v>
+        <v>Факел</v>
       </c>
       <c r="J35" t="str">
         <v>no_pic</v>
       </c>
       <c r="K35" t="str">
-        <v>Ротор</v>
+        <v>Акрон</v>
       </c>
       <c r="L35" t="str">
         <v>no_pic</v>
       </c>
       <c r="M35" t="str">
-        <v>Сочи</v>
+        <v>Оренбург</v>
       </c>
       <c r="N35" t="str">
         <v>no_pic</v>
       </c>
       <c r="O35" t="str">
-        <v>Акрон</v>
+        <v>Нижний Новгород</v>
       </c>
       <c r="P35" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q35" t="str">
-        <v>Ахмат</v>
+        <v>Динамо Махачкала</v>
       </c>
       <c r="R35" t="str">
         <v/>
@@ -2679,58 +2679,58 @@
         <v>1</v>
       </c>
       <c r="B36" t="str">
-        <v>Чья эта эмблема?</v>
+        <v>Кто стал первым чемпионом российской Премьер-лиги после её создания?</v>
       </c>
       <c r="C36" t="str">
-        <v>logo_ks</v>
+        <v>no_pic</v>
       </c>
       <c r="D36" t="str">
-        <v/>
+        <v>В 2002 году «Локомотив» стал первым чемпионом новой Премьер-лиги.</v>
       </c>
       <c r="E36" t="str">
-        <v>logo_ks</v>
+        <v>no_pic</v>
       </c>
       <c r="F36" t="str">
         <v>no_pic</v>
       </c>
       <c r="G36" t="str">
-        <v>Крылья Советов</v>
+        <v>«Локомотив»</v>
       </c>
       <c r="H36" t="str">
         <v>no_pic</v>
       </c>
       <c r="I36" t="str">
-        <v>Факел</v>
+        <v>«Спартак»</v>
       </c>
       <c r="J36" t="str">
         <v>no_pic</v>
       </c>
       <c r="K36" t="str">
-        <v>Акрон</v>
+        <v>ЦСКА</v>
       </c>
       <c r="L36" t="str">
         <v>no_pic</v>
       </c>
       <c r="M36" t="str">
-        <v>Оренбург</v>
+        <v>«Зенит»</v>
       </c>
       <c r="N36" t="str">
         <v>no_pic</v>
       </c>
       <c r="O36" t="str">
-        <v>Нижний Новгород</v>
+        <v>«Динамо»</v>
       </c>
       <c r="P36" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q36" t="str">
-        <v>Динамо Махачкала</v>
+        <v>«Рубин»</v>
       </c>
       <c r="R36" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="S36" t="str">
-        <v/>
+        <v>«Торпедо»</v>
       </c>
       <c r="T36" t="str">
         <v/>
@@ -2744,13 +2744,13 @@
         <v>1</v>
       </c>
       <c r="B37" t="str">
-        <v>Кто стал первым чемпионом российской Премьер-лиги после её создания?</v>
+        <v>Кого «Локомотив» победил в знаменитом Золотом матче 2002 года?</v>
       </c>
       <c r="C37" t="str">
         <v>no_pic</v>
       </c>
       <c r="D37" t="str">
-        <v>В 2002 году «Локомотив» стал первым чемпионом новой Премьер-лиги.</v>
+        <v>Чемпионство определилось в дополнительном Золотом матче между «Локомотивом» и ЦСКА.</v>
       </c>
       <c r="E37" t="str">
         <v>no_pic</v>
@@ -2759,7 +2759,7 @@
         <v>no_pic</v>
       </c>
       <c r="G37" t="str">
-        <v>«Локомотив»</v>
+        <v>ЦСКА</v>
       </c>
       <c r="H37" t="str">
         <v>no_pic</v>
@@ -2771,31 +2771,31 @@
         <v>no_pic</v>
       </c>
       <c r="K37" t="str">
-        <v>ЦСКА</v>
+        <v>«Зенит»</v>
       </c>
       <c r="L37" t="str">
         <v>no_pic</v>
       </c>
       <c r="M37" t="str">
-        <v>«Зенит»</v>
+        <v>«Динамо»</v>
       </c>
       <c r="N37" t="str">
         <v>no_pic</v>
       </c>
       <c r="O37" t="str">
-        <v>«Динамо»</v>
+        <v>«Крылья Советов»</v>
       </c>
       <c r="P37" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q37" t="str">
-        <v>«Рубин»</v>
+        <v>«Торпедо»</v>
       </c>
       <c r="R37" t="str">
         <v>no_pic</v>
       </c>
       <c r="S37" t="str">
-        <v>«Торпедо»</v>
+        <v>«Ротор»</v>
       </c>
       <c r="T37" t="str">
         <v/>
@@ -2809,13 +2809,13 @@
         <v>1</v>
       </c>
       <c r="B38" t="str">
-        <v>Кого «Локомотив» победил в знаменитом Золотом матче 2002 года?</v>
+        <v>Где прошёл первый официальный футбольный матч в Российской империи?</v>
       </c>
       <c r="C38" t="str">
         <v>no_pic</v>
       </c>
       <c r="D38" t="str">
-        <v>Чемпионство определилось в дополнительном Золотом матче между «Локомотивом» и ЦСКА.</v>
+        <v>Историческая встреча состоялась 24 октября 1897 года в Санкт-Петербурге.</v>
       </c>
       <c r="E38" t="str">
         <v>no_pic</v>
@@ -2824,43 +2824,43 @@
         <v>no_pic</v>
       </c>
       <c r="G38" t="str">
-        <v>ЦСКА</v>
+        <v>Санкт-Петербурге</v>
       </c>
       <c r="H38" t="str">
         <v>no_pic</v>
       </c>
       <c r="I38" t="str">
-        <v>«Спартак»</v>
+        <v>Москве</v>
       </c>
       <c r="J38" t="str">
         <v>no_pic</v>
       </c>
       <c r="K38" t="str">
-        <v>«Зенит»</v>
+        <v>Киеве</v>
       </c>
       <c r="L38" t="str">
         <v>no_pic</v>
       </c>
       <c r="M38" t="str">
-        <v>«Динамо»</v>
+        <v>Одессе</v>
       </c>
       <c r="N38" t="str">
         <v>no_pic</v>
       </c>
       <c r="O38" t="str">
-        <v>«Крылья Советов»</v>
+        <v>Харькове</v>
       </c>
       <c r="P38" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q38" t="str">
-        <v>«Торпедо»</v>
+        <v>Тифлисе</v>
       </c>
       <c r="R38" t="str">
         <v>no_pic</v>
       </c>
       <c r="S38" t="str">
-        <v>«Ротор»</v>
+        <v>Риге</v>
       </c>
       <c r="T38" t="str">
         <v/>
@@ -2874,13 +2874,13 @@
         <v>1</v>
       </c>
       <c r="B39" t="str">
-        <v>Где прошёл первый официальный футбольный матч в Российской империи?</v>
+        <v>Какая сборная нанесла Российской империи знаменитое поражение 0:16 на Олимпиаде 1912 года?</v>
       </c>
       <c r="C39" t="str">
         <v>no_pic</v>
       </c>
       <c r="D39" t="str">
-        <v>Историческая встреча состоялась 24 октября 1897 года в Санкт-Петербурге.</v>
+        <v>Разгром от Германии остаётся одним из самых известных эпизодов ранней истории российского футбола.</v>
       </c>
       <c r="E39" t="str">
         <v>no_pic</v>
@@ -2889,43 +2889,43 @@
         <v>no_pic</v>
       </c>
       <c r="G39" t="str">
-        <v>Санкт-Петербурге</v>
+        <v>Германия</v>
       </c>
       <c r="H39" t="str">
         <v>no_pic</v>
       </c>
       <c r="I39" t="str">
-        <v>Москве</v>
+        <v>Швеция</v>
       </c>
       <c r="J39" t="str">
         <v>no_pic</v>
       </c>
       <c r="K39" t="str">
-        <v>Киеве</v>
+        <v>Финляндия</v>
       </c>
       <c r="L39" t="str">
         <v>no_pic</v>
       </c>
       <c r="M39" t="str">
-        <v>Одессе</v>
+        <v>Венгрия</v>
       </c>
       <c r="N39" t="str">
         <v>no_pic</v>
       </c>
       <c r="O39" t="str">
-        <v>Харькове</v>
+        <v>Норвегия</v>
       </c>
       <c r="P39" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q39" t="str">
-        <v>Тифлисе</v>
+        <v>Дания</v>
       </c>
       <c r="R39" t="str">
         <v>no_pic</v>
       </c>
       <c r="S39" t="str">
-        <v>Риге</v>
+        <v>Австрия</v>
       </c>
       <c r="T39" t="str">
         <v/>
@@ -2939,13 +2939,13 @@
         <v>1</v>
       </c>
       <c r="B40" t="str">
-        <v>Какая сборная нанесла Российской империи знаменитое поражение 0:16 на Олимпиаде 1912 года?</v>
+        <v>В каком году сборная СССР стала чемпионом Европы?</v>
       </c>
       <c r="C40" t="str">
         <v>no_pic</v>
       </c>
       <c r="D40" t="str">
-        <v>Разгром от Германии остаётся одним из самых известных эпизодов ранней истории российского футбола.</v>
+        <v>Победа на первом в истории Кубке европейских наций 1960 года стала главным континентальным титулом сборной СССР.</v>
       </c>
       <c r="E40" t="str">
         <v>no_pic</v>
@@ -2954,43 +2954,43 @@
         <v>no_pic</v>
       </c>
       <c r="G40" t="str">
-        <v>Германия</v>
+        <v>1960</v>
       </c>
       <c r="H40" t="str">
         <v>no_pic</v>
       </c>
       <c r="I40" t="str">
-        <v>Швеция</v>
+        <v>1956</v>
       </c>
       <c r="J40" t="str">
         <v>no_pic</v>
       </c>
       <c r="K40" t="str">
-        <v>Финляндия</v>
+        <v>1964</v>
       </c>
       <c r="L40" t="str">
         <v>no_pic</v>
       </c>
       <c r="M40" t="str">
-        <v>Венгрия</v>
+        <v>1966</v>
       </c>
       <c r="N40" t="str">
         <v>no_pic</v>
       </c>
       <c r="O40" t="str">
-        <v>Норвегия</v>
+        <v>1968</v>
       </c>
       <c r="P40" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q40" t="str">
-        <v>Дания</v>
+        <v>1972</v>
       </c>
       <c r="R40" t="str">
         <v>no_pic</v>
       </c>
       <c r="S40" t="str">
-        <v>Австрия</v>
+        <v>1988</v>
       </c>
       <c r="T40" t="str">
         <v/>
@@ -3004,13 +3004,13 @@
         <v>1</v>
       </c>
       <c r="B41" t="str">
-        <v>В каком году сборная СССР стала чемпионом Европы?</v>
+        <v>В каком году «Зенит» впервые стал чемпионом СССР?</v>
       </c>
       <c r="C41" t="str">
         <v>no_pic</v>
       </c>
       <c r="D41" t="str">
-        <v>Победа на первом в истории Кубке европейских наций 1960 года стала главным континентальным титулом сборной СССР.</v>
+        <v>Единственное советское чемпионство ленинградского «Зенита» пришлось на 1984 год.</v>
       </c>
       <c r="E41" t="str">
         <v>no_pic</v>
@@ -3019,43 +3019,43 @@
         <v>no_pic</v>
       </c>
       <c r="G41" t="str">
-        <v>1960</v>
+        <v>1984</v>
       </c>
       <c r="H41" t="str">
         <v>no_pic</v>
       </c>
       <c r="I41" t="str">
-        <v>1956</v>
+        <v>1978</v>
       </c>
       <c r="J41" t="str">
         <v>no_pic</v>
       </c>
       <c r="K41" t="str">
-        <v>1964</v>
+        <v>1980</v>
       </c>
       <c r="L41" t="str">
         <v>no_pic</v>
       </c>
       <c r="M41" t="str">
-        <v>1966</v>
+        <v>1982</v>
       </c>
       <c r="N41" t="str">
         <v>no_pic</v>
       </c>
       <c r="O41" t="str">
-        <v>1968</v>
+        <v>1986</v>
       </c>
       <c r="P41" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q41" t="str">
-        <v>1972</v>
+        <v>1988</v>
       </c>
       <c r="R41" t="str">
         <v>no_pic</v>
       </c>
       <c r="S41" t="str">
-        <v>1988</v>
+        <v>1990</v>
       </c>
       <c r="T41" t="str">
         <v/>
@@ -3069,13 +3069,13 @@
         <v>1</v>
       </c>
       <c r="B42" t="str">
-        <v>В каком году «Зенит» впервые стал чемпионом СССР?</v>
+        <v>Какой клуб является самым титулованным в истории чемпионата СССР?</v>
       </c>
       <c r="C42" t="str">
         <v>no_pic</v>
       </c>
       <c r="D42" t="str">
-        <v>Единственное советское чемпионство ленинградского «Зенита» пришлось на 1984 год.</v>
+        <v>Киевское «Динамо» выиграло чемпионат СССР 13 раз, опередив «Спартак» с 12 титулами.</v>
       </c>
       <c r="E42" t="str">
         <v>no_pic</v>
@@ -3084,43 +3084,43 @@
         <v>no_pic</v>
       </c>
       <c r="G42" t="str">
-        <v>1984</v>
+        <v>«Динамо» Киев</v>
       </c>
       <c r="H42" t="str">
         <v>no_pic</v>
       </c>
       <c r="I42" t="str">
-        <v>1978</v>
+        <v>«Спартак» Москва</v>
       </c>
       <c r="J42" t="str">
         <v>no_pic</v>
       </c>
       <c r="K42" t="str">
-        <v>1980</v>
+        <v>«Динамо» Москва</v>
       </c>
       <c r="L42" t="str">
         <v>no_pic</v>
       </c>
       <c r="M42" t="str">
-        <v>1982</v>
+        <v>ЦСКА</v>
       </c>
       <c r="N42" t="str">
         <v>no_pic</v>
       </c>
       <c r="O42" t="str">
-        <v>1986</v>
+        <v>«Торпедо» Москва</v>
       </c>
       <c r="P42" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q42" t="str">
-        <v>1988</v>
+        <v>«Динамо» Тбилиси</v>
       </c>
       <c r="R42" t="str">
         <v>no_pic</v>
       </c>
       <c r="S42" t="str">
-        <v>1990</v>
+        <v>«Зенит» Ленинград</v>
       </c>
       <c r="T42" t="str">
         <v/>
@@ -3134,13 +3134,13 @@
         <v>1</v>
       </c>
       <c r="B43" t="str">
-        <v>Какой клуб является самым титулованным в истории чемпионата СССР?</v>
+        <v>Какой советский клуб первым в истории выиграл европейский клубный трофей?</v>
       </c>
       <c r="C43" t="str">
         <v>no_pic</v>
       </c>
       <c r="D43" t="str">
-        <v>Киевское «Динамо» выиграло чемпионат СССР 13 раз, опередив «Спартак» с 12 титулами.</v>
+        <v>В 1975 году киевское «Динамо» первым из советских клубов завоевало Кубок обладателей кубков.</v>
       </c>
       <c r="E43" t="str">
         <v>no_pic</v>
@@ -3167,25 +3167,25 @@
         <v>no_pic</v>
       </c>
       <c r="M43" t="str">
+        <v>«Динамо» Тбилиси</v>
+      </c>
+      <c r="N43" t="str">
+        <v>no_pic</v>
+      </c>
+      <c r="O43" t="str">
         <v>ЦСКА</v>
       </c>
-      <c r="N43" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="O43" t="str">
-        <v>«Торпедо» Москва</v>
-      </c>
       <c r="P43" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q43" t="str">
-        <v>«Динамо» Тбилиси</v>
+        <v>«Зенит»</v>
       </c>
       <c r="R43" t="str">
         <v>no_pic</v>
       </c>
       <c r="S43" t="str">
-        <v>«Зенит» Ленинград</v>
+        <v>«Торпедо»</v>
       </c>
       <c r="T43" t="str">
         <v/>
@@ -3199,13 +3199,13 @@
         <v>1</v>
       </c>
       <c r="B44" t="str">
-        <v>Какой советский клуб первым в истории выиграл европейский клубный трофей?</v>
+        <v>Под каким флагом сборная СНГ выступала на Евро-1992?</v>
       </c>
       <c r="C44" t="str">
         <v>no_pic</v>
       </c>
       <c r="D44" t="str">
-        <v>В 1975 году киевское «Динамо» первым из советских клубов завоевало Кубок обладателей кубков.</v>
+        <v>На Евро-1992 сборная СНГ играла под белым флагом с надписью C.I.S.</v>
       </c>
       <c r="E44" t="str">
         <v>no_pic</v>
@@ -3214,43 +3214,43 @@
         <v>no_pic</v>
       </c>
       <c r="G44" t="str">
-        <v>«Динамо» Киев</v>
+        <v>Под белым флагом с буквами C.I.S.</v>
       </c>
       <c r="H44" t="str">
         <v>no_pic</v>
       </c>
       <c r="I44" t="str">
-        <v>«Спартак» Москва</v>
+        <v>Под флагом СССР</v>
       </c>
       <c r="J44" t="str">
         <v>no_pic</v>
       </c>
       <c r="K44" t="str">
-        <v>«Динамо» Москва</v>
+        <v>Под флагом России</v>
       </c>
       <c r="L44" t="str">
         <v>no_pic</v>
       </c>
       <c r="M44" t="str">
-        <v>«Динамо» Тбилиси</v>
+        <v>Под флагом УЕФА</v>
       </c>
       <c r="N44" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="O44" t="str">
-        <v>ЦСКА</v>
+        <v/>
       </c>
       <c r="P44" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="Q44" t="str">
-        <v>«Зенит»</v>
+        <v/>
       </c>
       <c r="R44" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="S44" t="str">
-        <v>«Торпедо»</v>
+        <v/>
       </c>
       <c r="T44" t="str">
         <v/>
@@ -3264,13 +3264,13 @@
         <v>1</v>
       </c>
       <c r="B45" t="str">
-        <v>Под каким флагом сборная СНГ выступала на Евро-1992?</v>
+        <v>Кто тренировал сборную СНГ на Евро-1992?</v>
       </c>
       <c r="C45" t="str">
         <v>no_pic</v>
       </c>
       <c r="D45" t="str">
-        <v>На Евро-1992 сборная СНГ играла под белым флагом с надписью C.I.S.</v>
+        <v>Анатолий Бышовец возглавлял сначала сборную СССР, а затем сборную СНГ на Евро-1992.</v>
       </c>
       <c r="E45" t="str">
         <v>no_pic</v>
@@ -3279,25 +3279,25 @@
         <v>no_pic</v>
       </c>
       <c r="G45" t="str">
-        <v>Под белым флагом с буквами C.I.S.</v>
+        <v>Анатолий Бышовец</v>
       </c>
       <c r="H45" t="str">
         <v>no_pic</v>
       </c>
       <c r="I45" t="str">
-        <v>Под флагом СССР</v>
+        <v>Валерий Лобановский</v>
       </c>
       <c r="J45" t="str">
         <v>no_pic</v>
       </c>
       <c r="K45" t="str">
-        <v>Под флагом России</v>
+        <v>Олег Романцев</v>
       </c>
       <c r="L45" t="str">
         <v>no_pic</v>
       </c>
       <c r="M45" t="str">
-        <v>Под флагом УЕФА</v>
+        <v>Павел Садырин</v>
       </c>
       <c r="N45" t="str">
         <v/>
@@ -3329,13 +3329,13 @@
         <v>1</v>
       </c>
       <c r="B46" t="str">
-        <v>Кто тренировал сборную СНГ на Евро-1992?</v>
+        <v>Какой трофей стал первым в истории московского «Торпедо»?</v>
       </c>
       <c r="C46" t="str">
         <v>no_pic</v>
       </c>
       <c r="D46" t="str">
-        <v>Анатолий Бышовец возглавлял сначала сборную СССР, а затем сборную СНГ на Евро-1992.</v>
+        <v>Первый трофей «Торпедо» завоевало в 1949 году — Кубок СССР.</v>
       </c>
       <c r="E46" t="str">
         <v>no_pic</v>
@@ -3344,25 +3344,25 @@
         <v>no_pic</v>
       </c>
       <c r="G46" t="str">
-        <v>Анатолий Бышовец</v>
+        <v>Кубок СССР</v>
       </c>
       <c r="H46" t="str">
         <v>no_pic</v>
       </c>
       <c r="I46" t="str">
-        <v>Валерий Лобановский</v>
+        <v>Чемпионат СССР</v>
       </c>
       <c r="J46" t="str">
         <v>no_pic</v>
       </c>
       <c r="K46" t="str">
-        <v>Олег Романцев</v>
+        <v>Кубок России</v>
       </c>
       <c r="L46" t="str">
         <v>no_pic</v>
       </c>
       <c r="M46" t="str">
-        <v>Павел Садырин</v>
+        <v>Кубок Федерации СССР</v>
       </c>
       <c r="N46" t="str">
         <v/>
@@ -3394,13 +3394,13 @@
         <v>1</v>
       </c>
       <c r="B47" t="str">
-        <v>Какой трофей стал первым в истории московского «Торпедо»?</v>
+        <v>Это было? На Олимпиаде-1952 СССР уступал Югославии 1:5, но сравнял счёт — 5:5.</v>
       </c>
       <c r="C47" t="str">
         <v>no_pic</v>
       </c>
       <c r="D47" t="str">
-        <v>Первый трофей «Торпедо» завоевало в 1949 году — Кубок СССР.</v>
+        <v>За последние 15 минут советская команда отыграла четыре мяча и добилась переигровки.</v>
       </c>
       <c r="E47" t="str">
         <v>no_pic</v>
@@ -3409,25 +3409,25 @@
         <v>no_pic</v>
       </c>
       <c r="G47" t="str">
-        <v>Кубок СССР</v>
+        <v>Да</v>
       </c>
       <c r="H47" t="str">
         <v>no_pic</v>
       </c>
       <c r="I47" t="str">
-        <v>Чемпионат СССР</v>
+        <v>Нет</v>
       </c>
       <c r="J47" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="K47" t="str">
-        <v>Кубок России</v>
+        <v/>
       </c>
       <c r="L47" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="M47" t="str">
-        <v>Кубок Федерации СССР</v>
+        <v/>
       </c>
       <c r="N47" t="str">
         <v/>
@@ -3459,13 +3459,13 @@
         <v>1</v>
       </c>
       <c r="B48" t="str">
-        <v>Это было? На Олимпиаде-1952 СССР уступал Югославии 1:5, но сравнял счёт — 5:5.</v>
+        <v>Какой московский клуб в СССР был напрямую связан с автомобильным заводом ЗИЛ?</v>
       </c>
       <c r="C48" t="str">
         <v>no_pic</v>
       </c>
       <c r="D48" t="str">
-        <v>За последние 15 минут советская команда отыграла четыре мяча и добилась переигровки.</v>
+        <v>Игроки «Торпедо» формально числились работниками автозавода, позднее получившего имя ЗИЛ.</v>
       </c>
       <c r="E48" t="str">
         <v>no_pic</v>
@@ -3474,25 +3474,25 @@
         <v>no_pic</v>
       </c>
       <c r="G48" t="str">
-        <v>Да</v>
+        <v>«Торпедо»</v>
       </c>
       <c r="H48" t="str">
         <v>no_pic</v>
       </c>
       <c r="I48" t="str">
-        <v>Нет</v>
+        <v>«Динамо»</v>
       </c>
       <c r="J48" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="K48" t="str">
-        <v/>
+        <v>«Спартак»</v>
       </c>
       <c r="L48" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="M48" t="str">
-        <v/>
+        <v>«Локомотив»</v>
       </c>
       <c r="N48" t="str">
         <v/>
@@ -3524,13 +3524,13 @@
         <v>1</v>
       </c>
       <c r="B49" t="str">
-        <v>Какой московский клуб в СССР был напрямую связан с автомобильным заводом ЗИЛ?</v>
+        <v>Это было? Лев Яшин вошёл в топ-5 самого первого голосования за «Золотой мяч» в 1956 году.</v>
       </c>
       <c r="C49" t="str">
         <v>no_pic</v>
       </c>
       <c r="D49" t="str">
-        <v>Игроки «Торпедо» формально числились работниками автозавода, позднее получившего имя ЗИЛ.</v>
+        <v>В дебютном голосовании «Золотого мяча» Яшин занял пятое место.</v>
       </c>
       <c r="E49" t="str">
         <v>no_pic</v>
@@ -3539,25 +3539,25 @@
         <v>no_pic</v>
       </c>
       <c r="G49" t="str">
-        <v>«Торпедо»</v>
+        <v>Да</v>
       </c>
       <c r="H49" t="str">
         <v>no_pic</v>
       </c>
       <c r="I49" t="str">
-        <v>«Динамо»</v>
+        <v>Нет</v>
       </c>
       <c r="J49" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="K49" t="str">
-        <v>«Спартак»</v>
+        <v/>
       </c>
       <c r="L49" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="M49" t="str">
-        <v>«Локомотив»</v>
+        <v/>
       </c>
       <c r="N49" t="str">
         <v/>
@@ -3589,13 +3589,13 @@
         <v>1</v>
       </c>
       <c r="B50" t="str">
-        <v>Это было? Лев Яшин вошёл в топ-5 самого первого голосования за «Золотой мяч» в 1956 году.</v>
+        <v>Кто предложил Льву Яшину пустой чек после триумфа СССР на Евро-1960?</v>
       </c>
       <c r="C50" t="str">
         <v>no_pic</v>
       </c>
       <c r="D50" t="str">
-        <v>В дебютном голосовании «Золотого мяча» Яшин занял пятое место.</v>
+        <v>Президент «Реала» Сантьяго Бернабеу предложил Яшину вписать любую сумму, но вратарь отказался от перехода.</v>
       </c>
       <c r="E50" t="str">
         <v>no_pic</v>
@@ -3604,25 +3604,25 @@
         <v>no_pic</v>
       </c>
       <c r="G50" t="str">
-        <v>Да</v>
+        <v>Сантьяго Бернабеу</v>
       </c>
       <c r="H50" t="str">
         <v>no_pic</v>
       </c>
       <c r="I50" t="str">
-        <v>Нет</v>
+        <v>Альфредо Ди Стефано</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="K50" t="str">
-        <v/>
+        <v>Ференц Пушкаш</v>
       </c>
       <c r="L50" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="M50" t="str">
-        <v/>
+        <v>Мигель Муньос</v>
       </c>
       <c r="N50" t="str">
         <v/>
@@ -3654,13 +3654,13 @@
         <v>1</v>
       </c>
       <c r="B51" t="str">
-        <v>Кто предложил Льву Яшину пустой чек после триумфа СССР на Евро-1960?</v>
+        <v>Это было? «Торпедо» выиграло первый в новейшей истории Кубок России.</v>
       </c>
       <c r="C51" t="str">
         <v>no_pic</v>
       </c>
       <c r="D51" t="str">
-        <v>Президент «Реала» Сантьяго Бернабеу предложил Яшину вписать любую сумму, но вратарь отказался от перехода.</v>
+        <v>Московское «Торпедо» стало обладателем Кубка России 1993 года.</v>
       </c>
       <c r="E51" t="str">
         <v>no_pic</v>
@@ -3669,25 +3669,25 @@
         <v>no_pic</v>
       </c>
       <c r="G51" t="str">
-        <v>Сантьяго Бернабеу</v>
+        <v>Да</v>
       </c>
       <c r="H51" t="str">
         <v>no_pic</v>
       </c>
       <c r="I51" t="str">
-        <v>Альфредо Ди Стефано</v>
+        <v>Нет</v>
       </c>
       <c r="J51" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="K51" t="str">
-        <v>Ференц Пушкаш</v>
+        <v/>
       </c>
       <c r="L51" t="str">
-        <v>no_pic</v>
+        <v/>
       </c>
       <c r="M51" t="str">
-        <v>Мигель Муньос</v>
+        <v/>
       </c>
       <c r="N51" t="str">
         <v/>
@@ -3719,13 +3719,13 @@
         <v>1</v>
       </c>
       <c r="B52" t="str">
-        <v>Это было? «Торпедо» выиграло первый в новейшей истории Кубок России.</v>
+        <v>До какой стадии дошла сборная России на домашнем чемпионате мира 2018 года?</v>
       </c>
       <c r="C52" t="str">
         <v>no_pic</v>
       </c>
       <c r="D52" t="str">
-        <v>Московское «Торпедо» стало обладателем Кубка России 1993 года.</v>
+        <v>Россия прошла Испанию в 1/8 финала и остановилась в четвертьфинале после матча с Хорватией.</v>
       </c>
       <c r="E52" t="str">
         <v>no_pic</v>
@@ -3734,25 +3734,25 @@
         <v>no_pic</v>
       </c>
       <c r="G52" t="str">
-        <v>Да</v>
+        <v>До четвертьфинала</v>
       </c>
       <c r="H52" t="str">
         <v>no_pic</v>
       </c>
       <c r="I52" t="str">
-        <v>Нет</v>
+        <v>До 1/8 финала</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="K52" t="str">
-        <v/>
+        <v>До полуфинала</v>
       </c>
       <c r="L52" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="M52" t="str">
-        <v/>
+        <v>До финала</v>
       </c>
       <c r="N52" t="str">
         <v/>
@@ -3784,13 +3784,13 @@
         <v>1</v>
       </c>
       <c r="B53" t="str">
-        <v>До какой стадии дошла сборная России на домашнем чемпионате мира 2018 года?</v>
+        <v>Кого Россия обыграла 3:1 в четвертьфинале Евро-2008?</v>
       </c>
       <c r="C53" t="str">
         <v>no_pic</v>
       </c>
       <c r="D53" t="str">
-        <v>Россия прошла Испанию в 1/8 финала и остановилась в четвертьфинале после матча с Хорватией.</v>
+        <v>В Базеле Россия победила Нидерланды 3:1 в дополнительное время.</v>
       </c>
       <c r="E53" t="str">
         <v>no_pic</v>
@@ -3799,31 +3799,31 @@
         <v>no_pic</v>
       </c>
       <c r="G53" t="str">
-        <v>До четвертьфинала</v>
+        <v>Нидерланды</v>
       </c>
       <c r="H53" t="str">
         <v>no_pic</v>
       </c>
       <c r="I53" t="str">
-        <v>До 1/8 финала</v>
+        <v>Испанию</v>
       </c>
       <c r="J53" t="str">
         <v>no_pic</v>
       </c>
       <c r="K53" t="str">
-        <v>До полуфинала</v>
+        <v>Швецию</v>
       </c>
       <c r="L53" t="str">
         <v>no_pic</v>
       </c>
       <c r="M53" t="str">
-        <v>До финала</v>
+        <v>Германию</v>
       </c>
       <c r="N53" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="O53" t="str">
-        <v/>
+        <v>Хорватию</v>
       </c>
       <c r="P53" t="str">
         <v/>
@@ -3849,13 +3849,13 @@
         <v>1</v>
       </c>
       <c r="B54" t="str">
-        <v>Кого Россия обыграла 3:1 в четвертьфинале Евро-2008?</v>
+        <v>Какой европейский гранд «Зенит» разгромил 4:0 на пути в финал Кубка УЕФА-2008?</v>
       </c>
       <c r="C54" t="str">
         <v>no_pic</v>
       </c>
       <c r="D54" t="str">
-        <v>В Базеле Россия победила Нидерланды 3:1 в дополнительное время.</v>
+        <v>После 1:1 в Мюнхене «Зенит» победил «Баварию» в Петербурге 4:0.</v>
       </c>
       <c r="E54" t="str">
         <v>no_pic</v>
@@ -3864,31 +3864,31 @@
         <v>no_pic</v>
       </c>
       <c r="G54" t="str">
-        <v>Нидерланды</v>
+        <v>«Баварию»</v>
       </c>
       <c r="H54" t="str">
         <v>no_pic</v>
       </c>
       <c r="I54" t="str">
-        <v>Испанию</v>
+        <v>«Реал»</v>
       </c>
       <c r="J54" t="str">
         <v>no_pic</v>
       </c>
       <c r="K54" t="str">
-        <v>Швецию</v>
+        <v>«Милан»</v>
       </c>
       <c r="L54" t="str">
         <v>no_pic</v>
       </c>
       <c r="M54" t="str">
-        <v>Германию</v>
+        <v>«Интер»</v>
       </c>
       <c r="N54" t="str">
         <v>no_pic</v>
       </c>
       <c r="O54" t="str">
-        <v>Хорватию</v>
+        <v>«Ливерпуль»</v>
       </c>
       <c r="P54" t="str">
         <v/>
@@ -3914,13 +3914,13 @@
         <v>1</v>
       </c>
       <c r="B55" t="str">
-        <v>Какой европейский гранд «Зенит» разгромил 4:0 на пути в финал Кубка УЕФА-2008?</v>
+        <v>В каком испанском клубе Валерий Карпин играл вместе с Александром Мостовым?</v>
       </c>
       <c r="C55" t="str">
         <v>no_pic</v>
       </c>
       <c r="D55" t="str">
-        <v>После 1:1 в Мюнхене «Зенит» победил «Баварию» в Петербурге 4:0.</v>
+        <v>Карпин перешёл в «Сельту» в 1997 году, куда Мостовой перебрался годом ранее.</v>
       </c>
       <c r="E55" t="str">
         <v>no_pic</v>
@@ -3929,31 +3929,31 @@
         <v>no_pic</v>
       </c>
       <c r="G55" t="str">
-        <v>«Баварию»</v>
+        <v>«Сельта»</v>
       </c>
       <c r="H55" t="str">
         <v>no_pic</v>
       </c>
       <c r="I55" t="str">
-        <v>«Реал»</v>
+        <v>«Валенсия»</v>
       </c>
       <c r="J55" t="str">
         <v>no_pic</v>
       </c>
       <c r="K55" t="str">
-        <v>«Милан»</v>
+        <v>«Реал Сосьедад»</v>
       </c>
       <c r="L55" t="str">
         <v>no_pic</v>
       </c>
       <c r="M55" t="str">
-        <v>«Интер»</v>
+        <v>«Алавес»</v>
       </c>
       <c r="N55" t="str">
         <v>no_pic</v>
       </c>
       <c r="O55" t="str">
-        <v>«Ливерпуль»</v>
+        <v>«Севилья»</v>
       </c>
       <c r="P55" t="str">
         <v/>
@@ -3979,13 +3979,13 @@
         <v>1</v>
       </c>
       <c r="B56" t="str">
-        <v>В каком испанском клубе Валерий Карпин играл вместе с Александром Мостовым?</v>
+        <v>Каким видом спорта, кроме футбола, серьёзно занимался Лев Яшин?</v>
       </c>
       <c r="C56" t="str">
         <v>no_pic</v>
       </c>
       <c r="D56" t="str">
-        <v>Карпин перешёл в «Сельту» в 1997 году, куда Мостовой перебрался годом ранее.</v>
+        <v>В начале 1950-х Яшин выступал за хоккейное «Динамо» и даже завоевал трофей.</v>
       </c>
       <c r="E56" t="str">
         <v>no_pic</v>
@@ -3994,31 +3994,31 @@
         <v>no_pic</v>
       </c>
       <c r="G56" t="str">
-        <v>«Сельта»</v>
+        <v>Хоккеем</v>
       </c>
       <c r="H56" t="str">
         <v>no_pic</v>
       </c>
       <c r="I56" t="str">
-        <v>«Валенсия»</v>
+        <v>Баскетболом</v>
       </c>
       <c r="J56" t="str">
         <v>no_pic</v>
       </c>
       <c r="K56" t="str">
-        <v>«Реал Сосьедад»</v>
+        <v>Волейболом</v>
       </c>
       <c r="L56" t="str">
         <v>no_pic</v>
       </c>
       <c r="M56" t="str">
-        <v>«Алавес»</v>
+        <v>Боксом</v>
       </c>
       <c r="N56" t="str">
         <v>no_pic</v>
       </c>
       <c r="O56" t="str">
-        <v>«Севилья»</v>
+        <v>Хоккеем с мячом</v>
       </c>
       <c r="P56" t="str">
         <v/>
@@ -4044,13 +4044,13 @@
         <v>1</v>
       </c>
       <c r="B57" t="str">
-        <v>Каким видом спорта, кроме футбола, серьёзно занимался Лев Яшин?</v>
+        <v>Перед каким чемпионатом мира разгорелся скандал с «Письмом четырнадцати»?</v>
       </c>
       <c r="C57" t="str">
         <v>no_pic</v>
       </c>
       <c r="D57" t="str">
-        <v>В начале 1950-х Яшин выступал за хоккейное «Динамо» и даже завоевал трофей.</v>
+        <v>Письмо было написано в 1993 году накануне подготовки сборной России к чемпионату мира 1994 года.</v>
       </c>
       <c r="E57" t="str">
         <v>no_pic</v>
@@ -4059,31 +4059,31 @@
         <v>no_pic</v>
       </c>
       <c r="G57" t="str">
-        <v>Хоккеем</v>
+        <v>ЧМ-1994</v>
       </c>
       <c r="H57" t="str">
         <v>no_pic</v>
       </c>
       <c r="I57" t="str">
-        <v>Баскетболом</v>
+        <v>ЧМ-1990</v>
       </c>
       <c r="J57" t="str">
         <v>no_pic</v>
       </c>
       <c r="K57" t="str">
-        <v>Волейболом</v>
+        <v>ЧМ-1998</v>
       </c>
       <c r="L57" t="str">
         <v>no_pic</v>
       </c>
       <c r="M57" t="str">
-        <v>Боксом</v>
+        <v>ЧМ-2002</v>
       </c>
       <c r="N57" t="str">
         <v>no_pic</v>
       </c>
       <c r="O57" t="str">
-        <v>Хоккеем с мячом</v>
+        <v>ЧМ-2006</v>
       </c>
       <c r="P57" t="str">
         <v/>
@@ -4109,13 +4109,13 @@
         <v>1</v>
       </c>
       <c r="B58" t="str">
-        <v>Перед каким чемпионатом мира разгорелся скандал с «Письмом четырнадцати»?</v>
+        <v>Кто был тренером сборной России на ЧЕ-1996?</v>
       </c>
       <c r="C58" t="str">
         <v>no_pic</v>
       </c>
       <c r="D58" t="str">
-        <v>Письмо было написано в 1993 году накануне подготовки сборной России к чемпионату мира 1994 года.</v>
+        <v>На Евро-1996 сборной России руководил Олег Романцев.</v>
       </c>
       <c r="E58" t="str">
         <v>no_pic</v>
@@ -4124,37 +4124,37 @@
         <v>no_pic</v>
       </c>
       <c r="G58" t="str">
-        <v>ЧМ-1994</v>
+        <v>Олег Романцев</v>
       </c>
       <c r="H58" t="str">
         <v>no_pic</v>
       </c>
       <c r="I58" t="str">
-        <v>ЧМ-1990</v>
+        <v>Павел Садырин</v>
       </c>
       <c r="J58" t="str">
         <v>no_pic</v>
       </c>
       <c r="K58" t="str">
-        <v>ЧМ-1998</v>
+        <v>Георгий Ярцев</v>
       </c>
       <c r="L58" t="str">
         <v>no_pic</v>
       </c>
       <c r="M58" t="str">
-        <v>ЧМ-2002</v>
+        <v>Валерий Газзаев</v>
       </c>
       <c r="N58" t="str">
         <v>no_pic</v>
       </c>
       <c r="O58" t="str">
-        <v>ЧМ-2006</v>
+        <v>Гус Хиддинк</v>
       </c>
       <c r="P58" t="str">
-        <v/>
+        <v>no_pic</v>
       </c>
       <c r="Q58" t="str">
-        <v/>
+        <v>Анатолий Бышовец</v>
       </c>
       <c r="R58" t="str">
         <v/>
@@ -4174,13 +4174,13 @@
         <v>1</v>
       </c>
       <c r="B59" t="str">
-        <v>Кто был тренером сборной России на ЧЕ-1996?</v>
+        <v>Кто забил первый гол сборной России на ЧМ-2002?</v>
       </c>
       <c r="C59" t="str">
         <v>no_pic</v>
       </c>
       <c r="D59" t="str">
-        <v>На Евро-1996 сборной России руководил Олег Романцев.</v>
+        <v>В первом матче с Тунисом счёт открыл Егор Титов.</v>
       </c>
       <c r="E59" t="str">
         <v>no_pic</v>
@@ -4189,37 +4189,37 @@
         <v>no_pic</v>
       </c>
       <c r="G59" t="str">
-        <v>Олег Романцев</v>
+        <v>Егор Титов</v>
       </c>
       <c r="H59" t="str">
         <v>no_pic</v>
       </c>
       <c r="I59" t="str">
-        <v>Павел Садырин</v>
+        <v>Валерий Карпин</v>
       </c>
       <c r="J59" t="str">
         <v>no_pic</v>
       </c>
       <c r="K59" t="str">
-        <v>Георгий Ярцев</v>
+        <v>Дмитрий Сычёв</v>
       </c>
       <c r="L59" t="str">
         <v>no_pic</v>
       </c>
       <c r="M59" t="str">
-        <v>Валерий Газзаев</v>
+        <v>Александр Кержаков</v>
       </c>
       <c r="N59" t="str">
         <v>no_pic</v>
       </c>
       <c r="O59" t="str">
-        <v>Гус Хиддинк</v>
+        <v>Владимир Бесчастных</v>
       </c>
       <c r="P59" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q59" t="str">
-        <v>Анатолий Бышовец</v>
+        <v>Александр Мостовой</v>
       </c>
       <c r="R59" t="str">
         <v/>
@@ -4239,13 +4239,13 @@
         <v>1</v>
       </c>
       <c r="B60" t="str">
-        <v>Кто забил первый гол сборной России на ЧМ-2002?</v>
+        <v>Какой испанский клуб стал первым в карьере Валерия Карпина?</v>
       </c>
       <c r="C60" t="str">
         <v>no_pic</v>
       </c>
       <c r="D60" t="str">
-        <v>В первом матче с Тунисом счёт открыл Егор Титов.</v>
+        <v>После «Спартака» Карпин уехал в Испанию и перешёл в «Реал Сосьедад».</v>
       </c>
       <c r="E60" t="str">
         <v>no_pic</v>
@@ -4254,37 +4254,37 @@
         <v>no_pic</v>
       </c>
       <c r="G60" t="str">
-        <v>Егор Титов</v>
+        <v>Реал Сосьедад</v>
       </c>
       <c r="H60" t="str">
         <v>no_pic</v>
       </c>
       <c r="I60" t="str">
-        <v>Валерий Карпин</v>
+        <v>Сельта</v>
       </c>
       <c r="J60" t="str">
         <v>no_pic</v>
       </c>
       <c r="K60" t="str">
-        <v>Дмитрий Сычёв</v>
+        <v>Валенсия</v>
       </c>
       <c r="L60" t="str">
         <v>no_pic</v>
       </c>
       <c r="M60" t="str">
-        <v>Александр Кержаков</v>
+        <v>Депортиво</v>
       </c>
       <c r="N60" t="str">
         <v>no_pic</v>
       </c>
       <c r="O60" t="str">
-        <v>Владимир Бесчастных</v>
+        <v>Севилья</v>
       </c>
       <c r="P60" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q60" t="str">
-        <v>Александр Мостовой</v>
+        <v>Вильярреал</v>
       </c>
       <c r="R60" t="str">
         <v/>
@@ -4304,13 +4304,13 @@
         <v>1</v>
       </c>
       <c r="B61" t="str">
-        <v>Какой испанский клуб стал первым в карьере Валерия Карпина?</v>
+        <v>Какой клуб становился чемпионом СССР 11 раз?</v>
       </c>
       <c r="C61" t="str">
         <v>no_pic</v>
       </c>
       <c r="D61" t="str">
-        <v>После «Спартака» Карпин уехал в Испанию и перешёл в «Реал Сосьедад».</v>
+        <v>Московское «Динамо» выиграло 11 чемпионатов СССР.</v>
       </c>
       <c r="E61" t="str">
         <v>no_pic</v>
@@ -4319,37 +4319,37 @@
         <v>no_pic</v>
       </c>
       <c r="G61" t="str">
-        <v>Реал Сосьедад</v>
+        <v>Динамо Москва</v>
       </c>
       <c r="H61" t="str">
         <v>no_pic</v>
       </c>
       <c r="I61" t="str">
-        <v>Сельта</v>
+        <v>Спартак Москва</v>
       </c>
       <c r="J61" t="str">
         <v>no_pic</v>
       </c>
       <c r="K61" t="str">
-        <v>Валенсия</v>
+        <v>ЦСКА</v>
       </c>
       <c r="L61" t="str">
         <v>no_pic</v>
       </c>
       <c r="M61" t="str">
-        <v>Депортиво</v>
+        <v>Торпедо Москва</v>
       </c>
       <c r="N61" t="str">
         <v>no_pic</v>
       </c>
       <c r="O61" t="str">
-        <v>Севилья</v>
+        <v>Локомотив Москва</v>
       </c>
       <c r="P61" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q61" t="str">
-        <v>Вильярреал</v>
+        <v>Динамо Киев</v>
       </c>
       <c r="R61" t="str">
         <v/>
@@ -4369,13 +4369,13 @@
         <v>1</v>
       </c>
       <c r="B62" t="str">
-        <v>Какой клуб становился чемпионом СССР 11 раз?</v>
+        <v>Кто был капитаном ЦСКА в финале Кубка УЕФА-2005?</v>
       </c>
       <c r="C62" t="str">
         <v>no_pic</v>
       </c>
       <c r="D62" t="str">
-        <v>Московское «Динамо» выиграло 11 чемпионатов СССР.</v>
+        <v>Капитаном ЦСКА в победном еврокубковом походе был Сергей Игнашевич.</v>
       </c>
       <c r="E62" t="str">
         <v>no_pic</v>
@@ -4384,37 +4384,37 @@
         <v>no_pic</v>
       </c>
       <c r="G62" t="str">
-        <v>Динамо Москва</v>
+        <v>Сергей Игнашевич</v>
       </c>
       <c r="H62" t="str">
         <v>no_pic</v>
       </c>
       <c r="I62" t="str">
-        <v>Спартак Москва</v>
+        <v>Игорь Акинфеев</v>
       </c>
       <c r="J62" t="str">
         <v>no_pic</v>
       </c>
       <c r="K62" t="str">
-        <v>ЦСКА</v>
+        <v>Евгений Алдонин</v>
       </c>
       <c r="L62" t="str">
         <v>no_pic</v>
       </c>
       <c r="M62" t="str">
-        <v>Торпедо Москва</v>
+        <v>Алексей Березуцкий</v>
       </c>
       <c r="N62" t="str">
         <v>no_pic</v>
       </c>
       <c r="O62" t="str">
-        <v>Локомотив Москва</v>
+        <v>Даниэл Карвальо</v>
       </c>
       <c r="P62" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q62" t="str">
-        <v>Динамо Киев</v>
+        <v>Ивица Олич</v>
       </c>
       <c r="R62" t="str">
         <v/>
@@ -4434,52 +4434,52 @@
         <v>1</v>
       </c>
       <c r="B63" t="str">
-        <v>Кто был капитаном ЦСКА в финале Кубка УЕФА-2005?</v>
+        <v>Кто этот футболист?</v>
       </c>
       <c r="C63" t="str">
-        <v>no_pic</v>
+        <v>lokomotiv_batrakov</v>
       </c>
       <c r="D63" t="str">
-        <v>Капитаном ЦСКА в победном еврокубковом походе был Сергей Игнашевич.</v>
+        <v>На фото — Алексей Батраков, полузащитник «Локомотива».</v>
       </c>
       <c r="E63" t="str">
-        <v>no_pic</v>
+        <v>lokomotiv_batrakov</v>
       </c>
       <c r="F63" t="str">
         <v>no_pic</v>
       </c>
       <c r="G63" t="str">
-        <v>Сергей Игнашевич</v>
+        <v>Алексей Батраков</v>
       </c>
       <c r="H63" t="str">
         <v>no_pic</v>
       </c>
       <c r="I63" t="str">
-        <v>Игорь Акинфеев</v>
+        <v>Матвей Кисляк</v>
       </c>
       <c r="J63" t="str">
         <v>no_pic</v>
       </c>
       <c r="K63" t="str">
-        <v>Евгений Алдонин</v>
+        <v>Сергей Пиняев</v>
       </c>
       <c r="L63" t="str">
         <v>no_pic</v>
       </c>
       <c r="M63" t="str">
-        <v>Алексей Березуцкий</v>
+        <v>Иван Обляков</v>
       </c>
       <c r="N63" t="str">
         <v>no_pic</v>
       </c>
       <c r="O63" t="str">
-        <v>Даниэл Карвальо</v>
+        <v>Константин Тюкавин</v>
       </c>
       <c r="P63" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q63" t="str">
-        <v>Ивица Олич</v>
+        <v>Максим Глушенков</v>
       </c>
       <c r="R63" t="str">
         <v/>
@@ -4502,37 +4502,37 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C64" t="str">
-        <v>lokomotiv_batrakov</v>
+        <v>zs_sobolev</v>
       </c>
       <c r="D64" t="str">
-        <v>На фото — Алексей Батраков, полузащитник «Локомотива».</v>
+        <v>На фото — Александр Соболев.</v>
       </c>
       <c r="E64" t="str">
-        <v>lokomotiv_batrakov</v>
+        <v>zs_sobolev</v>
       </c>
       <c r="F64" t="str">
         <v>no_pic</v>
       </c>
       <c r="G64" t="str">
-        <v>Алексей Батраков</v>
+        <v>Александр Соболев</v>
       </c>
       <c r="H64" t="str">
         <v>no_pic</v>
       </c>
       <c r="I64" t="str">
-        <v>Матвей Кисляк</v>
+        <v>Артём Дзюба</v>
       </c>
       <c r="J64" t="str">
         <v>no_pic</v>
       </c>
       <c r="K64" t="str">
-        <v>Сергей Пиняев</v>
+        <v>Николай Комличенко</v>
       </c>
       <c r="L64" t="str">
         <v>no_pic</v>
       </c>
       <c r="M64" t="str">
-        <v>Иван Обляков</v>
+        <v>Иван Сергеев</v>
       </c>
       <c r="N64" t="str">
         <v>no_pic</v>
@@ -4544,7 +4544,7 @@
         <v>no_pic</v>
       </c>
       <c r="Q64" t="str">
-        <v>Максим Глушенков</v>
+        <v>Гамид Агаларов</v>
       </c>
       <c r="R64" t="str">
         <v/>
@@ -4567,49 +4567,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C65" t="str">
-        <v>zs_sobolev</v>
+        <v>spartak_maksimenko</v>
       </c>
       <c r="D65" t="str">
-        <v>На фото — Александр Соболев.</v>
+        <v>На фото — Александр Максименко, вратарь «Спартака».</v>
       </c>
       <c r="E65" t="str">
-        <v>zs_sobolev</v>
+        <v>spartak_maksimenko</v>
       </c>
       <c r="F65" t="str">
         <v>no_pic</v>
       </c>
       <c r="G65" t="str">
-        <v>Александр Соболев</v>
+        <v>Александр Максименко</v>
       </c>
       <c r="H65" t="str">
         <v>no_pic</v>
       </c>
       <c r="I65" t="str">
-        <v>Артём Дзюба</v>
+        <v>Игорь Акинфеев</v>
       </c>
       <c r="J65" t="str">
         <v>no_pic</v>
       </c>
       <c r="K65" t="str">
-        <v>Николай Комличенко</v>
+        <v>Андрей Лунёв</v>
       </c>
       <c r="L65" t="str">
         <v>no_pic</v>
       </c>
       <c r="M65" t="str">
-        <v>Иван Сергеев</v>
+        <v>Матвей Сафонов</v>
       </c>
       <c r="N65" t="str">
         <v>no_pic</v>
       </c>
       <c r="O65" t="str">
-        <v>Константин Тюкавин</v>
+        <v>Илья Лантратов</v>
       </c>
       <c r="P65" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q65" t="str">
-        <v>Гамид Агаларов</v>
+        <v>Евгений Латышонок</v>
       </c>
       <c r="R65" t="str">
         <v/>
@@ -4632,49 +4632,49 @@
         <v>Кто этот футболист?</v>
       </c>
       <c r="C66" t="str">
-        <v>spartak_maksimenko</v>
+        <v>lokomotiv_dzhikiya</v>
       </c>
       <c r="D66" t="str">
-        <v>На фото — Александр Максименко, вратарь «Спартака».</v>
+        <v>На фото — Георгий Джикия.</v>
       </c>
       <c r="E66" t="str">
-        <v>spartak_maksimenko</v>
+        <v>lokomotiv_dzhikiya</v>
       </c>
       <c r="F66" t="str">
         <v>no_pic</v>
       </c>
       <c r="G66" t="str">
-        <v>Александр Максименко</v>
+        <v>Георгий Джикия</v>
       </c>
       <c r="H66" t="str">
         <v>no_pic</v>
       </c>
       <c r="I66" t="str">
-        <v>Игорь Акинфеев</v>
+        <v>Игорь Дивеев</v>
       </c>
       <c r="J66" t="str">
         <v>no_pic</v>
       </c>
       <c r="K66" t="str">
-        <v>Андрей Лунёв</v>
+        <v>Максим Осипенко</v>
       </c>
       <c r="L66" t="str">
         <v>no_pic</v>
       </c>
       <c r="M66" t="str">
-        <v>Матвей Сафонов</v>
+        <v>Сергей Петров</v>
       </c>
       <c r="N66" t="str">
         <v>no_pic</v>
       </c>
       <c r="O66" t="str">
-        <v>Илья Лантратов</v>
+        <v>Роман Зобнин</v>
       </c>
       <c r="P66" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q66" t="str">
-        <v>Евгений Латышонок</v>
+        <v>Дмитрий Чистяков</v>
       </c>
       <c r="R66" t="str">
         <v/>
@@ -4694,52 +4694,52 @@
         <v>1</v>
       </c>
       <c r="B67" t="str">
-        <v>Кто этот футболист?</v>
+        <v>Какое название ранее носил ФК «Ростов»?</v>
       </c>
       <c r="C67" t="str">
-        <v>lokomotiv_dzhikiya</v>
+        <v>no_pic</v>
       </c>
       <c r="D67" t="str">
-        <v>На фото — Георгий Джикия.</v>
+        <v>До 2003 года клуб выступал под названием «Ростсельмаш».</v>
       </c>
       <c r="E67" t="str">
-        <v>lokomotiv_dzhikiya</v>
+        <v>no_pic</v>
       </c>
       <c r="F67" t="str">
         <v>no_pic</v>
       </c>
       <c r="G67" t="str">
-        <v>Георгий Джикия</v>
+        <v>Ростсельмаш</v>
       </c>
       <c r="H67" t="str">
         <v>no_pic</v>
       </c>
       <c r="I67" t="str">
-        <v>Игорь Дивеев</v>
+        <v>Ростовсельмаш</v>
       </c>
       <c r="J67" t="str">
         <v>no_pic</v>
       </c>
       <c r="K67" t="str">
-        <v>Максим Осипенко</v>
+        <v>Шахтёр</v>
       </c>
       <c r="L67" t="str">
         <v>no_pic</v>
       </c>
       <c r="M67" t="str">
-        <v>Сергей Петров</v>
+        <v>Пищевик</v>
       </c>
       <c r="N67" t="str">
         <v>no_pic</v>
       </c>
       <c r="O67" t="str">
-        <v>Роман Зобнин</v>
+        <v>Торпедо</v>
       </c>
       <c r="P67" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q67" t="str">
-        <v>Дмитрий Чистяков</v>
+        <v>Труд</v>
       </c>
       <c r="R67" t="str">
         <v/>
@@ -4759,13 +4759,13 @@
         <v>1</v>
       </c>
       <c r="B68" t="str">
-        <v>Какое название ранее носил ФК «Ростов»?</v>
+        <v>Какой известный бывший нападающий «Спартака» и сборной России тренировал «Родину»?</v>
       </c>
       <c r="C68" t="str">
         <v>no_pic</v>
       </c>
       <c r="D68" t="str">
-        <v>До 2003 года клуб выступал под названием «Ростсельмаш».</v>
+        <v>В 2024 году главным тренером «Родины» был Владимир Бесчастных.</v>
       </c>
       <c r="E68" t="str">
         <v>no_pic</v>
@@ -4774,37 +4774,37 @@
         <v>no_pic</v>
       </c>
       <c r="G68" t="str">
-        <v>Ростсельмаш</v>
+        <v>Владимир Бесчастных</v>
       </c>
       <c r="H68" t="str">
         <v>no_pic</v>
       </c>
       <c r="I68" t="str">
-        <v>Ростовсельмаш</v>
+        <v>Александр Мостовой</v>
       </c>
       <c r="J68" t="str">
         <v>no_pic</v>
       </c>
       <c r="K68" t="str">
-        <v>Шахтёр</v>
+        <v>Егор Титов</v>
       </c>
       <c r="L68" t="str">
         <v>no_pic</v>
       </c>
       <c r="M68" t="str">
-        <v>Пищевик</v>
+        <v>Дмитрий Аленичев</v>
       </c>
       <c r="N68" t="str">
         <v>no_pic</v>
       </c>
       <c r="O68" t="str">
-        <v>Торпедо</v>
+        <v>Андрей Тихонов</v>
       </c>
       <c r="P68" t="str">
         <v>no_pic</v>
       </c>
       <c r="Q68" t="str">
-        <v>Труд</v>
+        <v>Роман Павлюченко</v>
       </c>
       <c r="R68" t="str">
         <v/>
@@ -4816,77 +4816,12 @@
         <v/>
       </c>
       <c r="U68" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>1</v>
-      </c>
-      <c r="B69" t="str">
-        <v>Какой известный бывший нападающий «Спартака» и сборной России тренировал «Родину»?</v>
-      </c>
-      <c r="C69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="D69" t="str">
-        <v>В 2024 году главным тренером «Родины» был Владимир Бесчастных.</v>
-      </c>
-      <c r="E69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="F69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="G69" t="str">
-        <v>Владимир Бесчастных</v>
-      </c>
-      <c r="H69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="I69" t="str">
-        <v>Александр Мостовой</v>
-      </c>
-      <c r="J69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="K69" t="str">
-        <v>Егор Титов</v>
-      </c>
-      <c r="L69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="M69" t="str">
-        <v>Дмитрий Аленичев</v>
-      </c>
-      <c r="N69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="O69" t="str">
-        <v>Андрей Тихонов</v>
-      </c>
-      <c r="P69" t="str">
-        <v>no_pic</v>
-      </c>
-      <c r="Q69" t="str">
-        <v>Роман Павлюченко</v>
-      </c>
-      <c r="R69" t="str">
-        <v/>
-      </c>
-      <c r="S69" t="str">
-        <v/>
-      </c>
-      <c r="T69" t="str">
-        <v/>
-      </c>
-      <c r="U69" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>